<commit_message>
Big changes to whole thing
</commit_message>
<xml_diff>
--- a/inst/pipeline/MARMOT_Metadata.xlsx
+++ b/inst/pipeline/MARMOT_Metadata.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10209"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10608"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/peterleary/Desktop/FGCZ/MARMOT/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/peterleary/Desktop/FGCZ/MARMOT/inst/pipeline/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{55FF4185-5194-2C45-8321-E6CB151EE7B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{55A9E34B-C84E-4447-8A0F-97983FD61864}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3460" yWindow="2760" windowWidth="39400" windowHeight="21660" xr2:uid="{9C611E3C-4644-F449-9441-E60F328909FC}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="34560" windowHeight="20440" xr2:uid="{9C611E3C-4644-F449-9441-E60F328909FC}"/>
   </bookViews>
   <sheets>
     <sheet name="Pipeline Settings" sheetId="3" r:id="rId1"/>
@@ -22,11 +22,12 @@
     <definedName name="clusteringMethodToUse" localSheetId="3">Options!$A$1:$A$4</definedName>
     <definedName name="dimRedMethodToUse">Options!$C$1:$C$3</definedName>
     <definedName name="markersToClusterBy">Options!$B$1:$B$3</definedName>
+    <definedName name="qcDropdown">Options!$D$1:$D$3</definedName>
     <definedName name="runQC">Options!$D$1:$D$2</definedName>
     <definedName name="themeToUse">Options!$E$1:$E$5</definedName>
     <definedName name="viridisColour">Options!$F$1:$F$8</definedName>
   </definedNames>
-  <calcPr calcId="181029" iterateDelta="1E-4"/>
+  <calcPr calcId="181029" concurrentCalc="0"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -46,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="201" uniqueCount="150">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="200" uniqueCount="148">
   <si>
     <t>Conditions To Test</t>
   </si>
@@ -318,9 +319,6 @@
     <t>markersToDimRedBy</t>
   </si>
   <si>
-    <t>drCellCount</t>
-  </si>
-  <si>
     <t>runQC</t>
   </si>
   <si>
@@ -402,9 +400,6 @@
     <t>Choose whether to use the QC-cleaned FCS files.</t>
   </si>
   <si>
-    <t>Choose whether to run flowAI QC.</t>
-  </si>
-  <si>
     <t xml:space="preserve">Do you want to save lots of the figures as PDFs? </t>
   </si>
   <si>
@@ -474,18 +469,9 @@
     <t>~/Desktop/MARMOT/</t>
   </si>
   <si>
-    <t>Enter one or more of FR (flow rate), FS (signal acquisition), and FM (dynamic range), space separated.</t>
-  </si>
-  <si>
-    <t>FR FS</t>
-  </si>
-  <si>
     <t>Number of cells to take from each FCS file. Leave blank to include all cells (will make things slow).</t>
   </si>
   <si>
-    <t xml:space="preserve">Enter a number to downsample to when calculating DR plots. Leave blank to include all cells. </t>
-  </si>
-  <si>
     <t>Enter an amount of RAM per processor core. Marmot likes at least 6. Make sure nCores*ramPerCore is less than your total amount of RAM</t>
   </si>
   <si>
@@ -495,7 +481,16 @@
     <t>Select a ggplot theme to use. Marmots like prism.</t>
   </si>
   <si>
-    <t>metricsQC</t>
+    <t>None</t>
+  </si>
+  <si>
+    <t>PeacoQC</t>
+  </si>
+  <si>
+    <t>FlowAI</t>
+  </si>
+  <si>
+    <t>Choose whether to run QC, and if so, which method.</t>
   </si>
 </sst>
 </file>
@@ -999,8 +994,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{3586C4B2-ADB2-8944-8759-A59E39853E12}" name="Table1" displayName="Table1" ref="A1:C22" totalsRowShown="0" headerRowDxfId="8" dataDxfId="6" headerRowBorderDxfId="7" tableBorderDxfId="5" totalsRowBorderDxfId="4">
-  <autoFilter ref="A1:C22" xr:uid="{3586C4B2-ADB2-8944-8759-A59E39853E12}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{3586C4B2-ADB2-8944-8759-A59E39853E12}" name="Table1" displayName="Table1" ref="A1:C20" totalsRowShown="0" headerRowDxfId="8" dataDxfId="6" headerRowBorderDxfId="7" tableBorderDxfId="5" totalsRowBorderDxfId="4">
+  <autoFilter ref="A1:C20" xr:uid="{3586C4B2-ADB2-8944-8759-A59E39853E12}"/>
   <tableColumns count="3">
     <tableColumn id="1" xr3:uid="{6E5D9E7E-2965-C342-935C-46AFF40862A4}" name="Variable" dataDxfId="3"/>
     <tableColumn id="2" xr3:uid="{3651CB78-AF61-9F48-9271-E82C28D1865F}" name="Setting" dataDxfId="2"/>
@@ -1307,7 +1302,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9B6B5C96-224E-6D44-823C-9DBA67F761F0}">
-  <dimension ref="A1:C23"/>
+  <dimension ref="A1:C21"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="20.83203125" style="7" bestFit="1" customWidth="1"/>
@@ -1317,13 +1312,13 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A1" s="6" t="s">
+        <v>100</v>
+      </c>
+      <c r="B1" s="10" t="s">
         <v>101</v>
       </c>
-      <c r="B1" s="10" t="s">
+      <c r="C1" s="5" t="s">
         <v>102</v>
-      </c>
-      <c r="C1" s="5" t="s">
-        <v>103</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.2">
@@ -1334,7 +1329,7 @@
         <v>1000</v>
       </c>
       <c r="C2" s="13" t="s">
-        <v>144</v>
+        <v>140</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.2">
@@ -1342,10 +1337,10 @@
         <v>84</v>
       </c>
       <c r="B3" s="15" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C3" s="16" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.2">
@@ -1353,10 +1348,10 @@
         <v>85</v>
       </c>
       <c r="B4" s="15" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C4" s="16" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.2">
@@ -1364,10 +1359,10 @@
         <v>86</v>
       </c>
       <c r="B5" s="15" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="C5" s="16" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.2">
@@ -1378,7 +1373,7 @@
         <v>20</v>
       </c>
       <c r="C6" s="16" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.2">
@@ -1386,10 +1381,10 @@
         <v>88</v>
       </c>
       <c r="B7" s="18" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="C7" s="19" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.2">
@@ -1400,16 +1395,18 @@
         <v>47</v>
       </c>
       <c r="C8" s="19" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A9" s="17" t="s">
+      <c r="A9" s="20" t="s">
         <v>90</v>
       </c>
-      <c r="B9" s="18"/>
-      <c r="C9" s="19" t="s">
+      <c r="B9" s="21" t="s">
         <v>145</v>
+      </c>
+      <c r="C9" s="22" t="s">
+        <v>147</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.2">
@@ -1417,46 +1414,46 @@
         <v>91</v>
       </c>
       <c r="B10" s="21" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C10" s="22" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A11" s="20" t="s">
-        <v>149</v>
-      </c>
-      <c r="B11" s="21" t="s">
-        <v>143</v>
-      </c>
-      <c r="C11" s="22" t="s">
-        <v>142</v>
+      <c r="A11" s="23" t="s">
+        <v>92</v>
+      </c>
+      <c r="B11" s="24"/>
+      <c r="C11" s="25" t="s">
+        <v>135</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A12" s="20" t="s">
-        <v>92</v>
-      </c>
-      <c r="B12" s="21" t="b">
+      <c r="A12" s="23" t="s">
+        <v>93</v>
+      </c>
+      <c r="B12" s="24" t="b">
         <v>0</v>
       </c>
-      <c r="C12" s="22" t="s">
+      <c r="C12" s="25" t="s">
         <v>117</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A13" s="23" t="s">
-        <v>93</v>
-      </c>
-      <c r="B13" s="24"/>
+        <v>94</v>
+      </c>
+      <c r="B13" s="24" t="b">
+        <v>0</v>
+      </c>
       <c r="C13" s="25" t="s">
-        <v>137</v>
+        <v>118</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A14" s="23" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="B14" s="24" t="b">
         <v>1</v>
@@ -1467,10 +1464,10 @@
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A15" s="23" t="s">
-        <v>95</v>
-      </c>
-      <c r="B15" s="24" t="b">
-        <v>0</v>
+        <v>96</v>
+      </c>
+      <c r="B15" s="24">
+        <v>4</v>
       </c>
       <c r="C15" s="25" t="s">
         <v>120</v>
@@ -1478,85 +1475,63 @@
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A16" s="23" t="s">
-        <v>96</v>
-      </c>
-      <c r="B16" s="24" t="b">
-        <v>1</v>
+        <v>97</v>
+      </c>
+      <c r="B16" s="24">
+        <v>6</v>
       </c>
       <c r="C16" s="25" t="s">
-        <v>121</v>
+        <v>141</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A17" s="23" t="s">
-        <v>97</v>
-      </c>
-      <c r="B17" s="24">
-        <v>4</v>
+        <v>98</v>
+      </c>
+      <c r="B17" s="24" t="s">
+        <v>121</v>
       </c>
       <c r="C17" s="25" t="s">
-        <v>122</v>
+        <v>143</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A18" s="23" t="s">
-        <v>98</v>
-      </c>
-      <c r="B18" s="24">
-        <v>6</v>
+        <v>99</v>
+      </c>
+      <c r="B18" s="24" t="s">
+        <v>131</v>
       </c>
       <c r="C18" s="25" t="s">
-        <v>146</v>
+        <v>142</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A19" s="23" t="s">
-        <v>99</v>
-      </c>
-      <c r="B19" s="24" t="s">
-        <v>123</v>
-      </c>
-      <c r="C19" s="25" t="s">
-        <v>148</v>
+      <c r="A19" s="26" t="s">
+        <v>81</v>
+      </c>
+      <c r="B19" s="27" t="s">
+        <v>136</v>
+      </c>
+      <c r="C19" s="28" t="s">
+        <v>137</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A20" s="23" t="s">
-        <v>100</v>
-      </c>
-      <c r="B20" s="24" t="s">
-        <v>133</v>
-      </c>
-      <c r="C20" s="25" t="s">
-        <v>147</v>
+      <c r="A20" s="29" t="s">
+        <v>82</v>
+      </c>
+      <c r="B20" s="30" t="s">
+        <v>139</v>
+      </c>
+      <c r="C20" s="31" t="s">
+        <v>138</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A21" s="26" t="s">
-        <v>81</v>
-      </c>
-      <c r="B21" s="27" t="s">
-        <v>138</v>
-      </c>
-      <c r="C21" s="28" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A22" s="29" t="s">
-        <v>82</v>
-      </c>
-      <c r="B22" s="30" t="s">
-        <v>141</v>
-      </c>
-      <c r="C22" s="31" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A23" s="8"/>
-      <c r="B23" s="8"/>
-      <c r="C23" s="9"/>
+      <c r="A21" s="8"/>
+      <c r="B21" s="8"/>
+      <c r="C21" s="9"/>
     </row>
   </sheetData>
   <conditionalFormatting sqref="B3">
@@ -1570,7 +1545,7 @@
   </tableParts>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
-      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="10">
+      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="11">
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{9EAFFEB3-23DE-8247-B8FE-8F1F5C2CC03D}">
           <x14:formula1>
             <xm:f>Options!$B$1:$B$3</xm:f>
@@ -1587,7 +1562,43 @@
           <x14:formula1>
             <xm:f>Options!$D$1:$D$2</xm:f>
           </x14:formula1>
-          <xm:sqref>B10 B12</xm:sqref>
+          <xm:sqref>B10</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{EA79EA2F-903F-354F-BF4D-E09B45EA2C79}">
+          <x14:formula1>
+            <xm:f>Options!G1:G2</xm:f>
+          </x14:formula1>
+          <xm:sqref>B12</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{5D9B856C-01B5-4640-9249-FF510B93E1FC}">
+          <x14:formula1>
+            <xm:f>Options!G1:G2</xm:f>
+          </x14:formula1>
+          <xm:sqref>B13</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{93DD8684-4441-9741-BAB6-CBE45BFB25B6}">
+          <x14:formula1>
+            <xm:f>Options!G1:G2</xm:f>
+          </x14:formula1>
+          <xm:sqref>B14</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{EF0F4D8A-D969-2040-A7B2-4D843CC1D241}">
+          <x14:formula1>
+            <xm:f>Options!$E$1:$E$5</xm:f>
+          </x14:formula1>
+          <xm:sqref>B17</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{D6D0959A-58E3-6B40-9F0A-C50FD537F1F2}">
+          <x14:formula1>
+            <xm:f>Options!$F$1:$F$8</xm:f>
+          </x14:formula1>
+          <xm:sqref>B18</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{C81D77FB-D1A4-0B4C-B41A-E5791F351257}">
+          <x14:formula1>
+            <xm:f>Options!$D$1:$D$3</xm:f>
+          </x14:formula1>
+          <xm:sqref>B9</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{ED65EFD9-012C-8E42-BE3B-3B16546394D0}">
           <x14:formula1>
@@ -1600,36 +1611,6 @@
             <xm:f>Options!B1:B3</xm:f>
           </x14:formula1>
           <xm:sqref>B8</xm:sqref>
-        </x14:dataValidation>
-        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{EA79EA2F-903F-354F-BF4D-E09B45EA2C79}">
-          <x14:formula1>
-            <xm:f>Options!D1:D2</xm:f>
-          </x14:formula1>
-          <xm:sqref>B14</xm:sqref>
-        </x14:dataValidation>
-        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{5D9B856C-01B5-4640-9249-FF510B93E1FC}">
-          <x14:formula1>
-            <xm:f>Options!D1:D2</xm:f>
-          </x14:formula1>
-          <xm:sqref>B15</xm:sqref>
-        </x14:dataValidation>
-        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{93DD8684-4441-9741-BAB6-CBE45BFB25B6}">
-          <x14:formula1>
-            <xm:f>Options!D1:D2</xm:f>
-          </x14:formula1>
-          <xm:sqref>B16</xm:sqref>
-        </x14:dataValidation>
-        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{EF0F4D8A-D969-2040-A7B2-4D843CC1D241}">
-          <x14:formula1>
-            <xm:f>Options!$E$1:$E$5</xm:f>
-          </x14:formula1>
-          <xm:sqref>B19</xm:sqref>
-        </x14:dataValidation>
-        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{D6D0959A-58E3-6B40-9F0A-C50FD537F1F2}">
-          <x14:formula1>
-            <xm:f>Options!$F$1:$F$8</xm:f>
-          </x14:formula1>
-          <xm:sqref>B20</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -2189,98 +2170,107 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C1FFB7FD-CFF9-C444-B899-D3ED2BB2FB65}">
-  <dimension ref="A1:F8"/>
+  <dimension ref="A1:G8"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B1" t="s">
         <v>47</v>
       </c>
       <c r="C1" t="s">
-        <v>112</v>
-      </c>
-      <c r="D1" t="b">
+        <v>111</v>
+      </c>
+      <c r="D1" t="s">
+        <v>144</v>
+      </c>
+      <c r="E1" t="s">
+        <v>121</v>
+      </c>
+      <c r="F1" t="s">
+        <v>126</v>
+      </c>
+      <c r="G1" t="b">
         <v>1</v>
       </c>
-      <c r="E1" t="s">
-        <v>123</v>
-      </c>
-      <c r="F1" t="s">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B2" t="s">
         <v>48</v>
       </c>
       <c r="C2" t="s">
+        <v>112</v>
+      </c>
+      <c r="D2" t="s">
+        <v>146</v>
+      </c>
+      <c r="E2" t="s">
+        <v>122</v>
+      </c>
+      <c r="F2" t="s">
+        <v>127</v>
+      </c>
+      <c r="G2" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>105</v>
+      </c>
+      <c r="B3" t="s">
+        <v>108</v>
+      </c>
+      <c r="C3" t="s">
         <v>113</v>
       </c>
-      <c r="D2" t="b">
-        <v>0</v>
-      </c>
-      <c r="E2" t="s">
+      <c r="D3" t="s">
+        <v>145</v>
+      </c>
+      <c r="E3" t="s">
+        <v>123</v>
+      </c>
+      <c r="F3" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>106</v>
+      </c>
+      <c r="E4" t="s">
         <v>124</v>
       </c>
-      <c r="F2" t="s">
+      <c r="F4" t="s">
         <v>129</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A3" t="s">
-        <v>106</v>
-      </c>
-      <c r="B3" t="s">
-        <v>109</v>
-      </c>
-      <c r="C3" t="s">
-        <v>114</v>
-      </c>
-      <c r="E3" t="s">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="E5" t="s">
         <v>125</v>
       </c>
-      <c r="F3" t="s">
+      <c r="F5" t="s">
         <v>130</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A4" t="s">
-        <v>107</v>
-      </c>
-      <c r="E4" t="s">
-        <v>126</v>
-      </c>
-      <c r="F4" t="s">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="F6" t="s">
         <v>131</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="E5" t="s">
-        <v>127</v>
-      </c>
-      <c r="F5" t="s">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="F7" t="s">
         <v>132</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="F6" t="s">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="F8" t="s">
         <v>133</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="F7" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="F8" t="s">
-        <v>135</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Small fix to metadata file
</commit_message>
<xml_diff>
--- a/inst/pipeline/MARMOT_Metadata.xlsx
+++ b/inst/pipeline/MARMOT_Metadata.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/peterleary/Desktop/FGCZ/MARMOT/inst/pipeline/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{55A9E34B-C84E-4447-8A0F-97983FD61864}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4804170E-B5B7-964D-B12A-CEE8B411D298}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="34560" windowHeight="20440" xr2:uid="{9C611E3C-4644-F449-9441-E60F328909FC}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="34560" windowHeight="20440" activeTab="2" xr2:uid="{9C611E3C-4644-F449-9441-E60F328909FC}"/>
   </bookViews>
   <sheets>
     <sheet name="Pipeline Settings" sheetId="3" r:id="rId1"/>
@@ -1560,7 +1560,7 @@
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{85A5D0C9-C8F8-D240-8860-5596AC9A9FC7}">
           <x14:formula1>
-            <xm:f>Options!$D$1:$D$2</xm:f>
+            <xm:f>Options!$G$1:$G$2</xm:f>
           </x14:formula1>
           <xm:sqref>B10</xm:sqref>
         </x14:dataValidation>

</xml_diff>

<commit_message>
Having a pop at using ragg instead of cairo
</commit_message>
<xml_diff>
--- a/inst/pipeline/MARMOT_Metadata.xlsx
+++ b/inst/pipeline/MARMOT_Metadata.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/peterleary/Desktop/FGCZ/MARMOT/inst/pipeline/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{97C00055-F929-AA43-A5B6-F39FE1405A06}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7A15C0BD-4E38-4341-8994-938EC02661E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="34560" windowHeight="20440" xr2:uid="{9C611E3C-4644-F449-9441-E60F328909FC}"/>
+    <workbookView xWindow="8220" yWindow="12740" windowWidth="34560" windowHeight="20440" activeTab="2" xr2:uid="{9C611E3C-4644-F449-9441-E60F328909FC}"/>
   </bookViews>
   <sheets>
     <sheet name="Pipeline Settings" sheetId="3" r:id="rId1"/>
@@ -27,7 +27,7 @@
     <definedName name="themeToUse">Options!$E$1:$E$5</definedName>
     <definedName name="viridisColour">Options!$F$1:$F$8</definedName>
   </definedNames>
-  <calcPr calcId="181029" concurrentCalc="0"/>
+  <calcPr calcId="181029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -809,7 +809,17 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="9">
+  <dxfs count="10">
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -994,12 +1004,12 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{3586C4B2-ADB2-8944-8759-A59E39853E12}" name="Table1" displayName="Table1" ref="A1:C20" totalsRowShown="0" headerRowDxfId="8" dataDxfId="6" headerRowBorderDxfId="7" tableBorderDxfId="5" totalsRowBorderDxfId="4">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{3586C4B2-ADB2-8944-8759-A59E39853E12}" name="Table1" displayName="Table1" ref="A1:C20" totalsRowShown="0" headerRowDxfId="9" dataDxfId="7" headerRowBorderDxfId="8" tableBorderDxfId="6" totalsRowBorderDxfId="5">
   <autoFilter ref="A1:C20" xr:uid="{3586C4B2-ADB2-8944-8759-A59E39853E12}"/>
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{6E5D9E7E-2965-C342-935C-46AFF40862A4}" name="Variable" dataDxfId="3"/>
-    <tableColumn id="2" xr3:uid="{3651CB78-AF61-9F48-9271-E82C28D1865F}" name="Setting" dataDxfId="2"/>
-    <tableColumn id="3" xr3:uid="{9A550912-B61D-BA41-87DB-136B1A08B9E2}" name="Info" dataDxfId="1"/>
+    <tableColumn id="1" xr3:uid="{6E5D9E7E-2965-C342-935C-46AFF40862A4}" name="Variable" dataDxfId="4"/>
+    <tableColumn id="2" xr3:uid="{3651CB78-AF61-9F48-9271-E82C28D1865F}" name="Setting" dataDxfId="3"/>
+    <tableColumn id="3" xr3:uid="{9A550912-B61D-BA41-87DB-136B1A08B9E2}" name="Info" dataDxfId="2"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1535,7 +1545,7 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="B3">
-    <cfRule type="expression" dxfId="0" priority="1">
+    <cfRule type="expression" dxfId="1" priority="1">
       <formula>ISBLANK(A3)</formula>
     </cfRule>
   </conditionalFormatting>
@@ -2164,6 +2174,9 @@
     </row>
   </sheetData>
   <phoneticPr fontId="3" type="noConversion"/>
+  <conditionalFormatting sqref="B2:B12">
+    <cfRule type="duplicateValues" dxfId="0" priority="1"/>
+  </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Small fix to parallelisation
</commit_message>
<xml_diff>
--- a/inst/pipeline/MARMOT_Metadata.xlsx
+++ b/inst/pipeline/MARMOT_Metadata.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/peterleary/Desktop/FGCZ/MARMOT/inst/pipeline/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{68D31D6F-A187-A04F-A861-E6FCC8C4A7EF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AC30FBCE-4B68-5A40-9C77-914E8E9744AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="7920" yWindow="6380" windowWidth="34560" windowHeight="20440" activeTab="1" xr2:uid="{9C611E3C-4644-F449-9441-E60F328909FC}"/>
+    <workbookView xWindow="15660" yWindow="4620" windowWidth="34560" windowHeight="20440" activeTab="1" xr2:uid="{9C611E3C-4644-F449-9441-E60F328909FC}"/>
   </bookViews>
   <sheets>
     <sheet name="Pipeline Settings" sheetId="3" r:id="rId1"/>
@@ -47,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="200" uniqueCount="148">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="206" uniqueCount="154">
   <si>
     <t>Conditions To Test</t>
   </si>
@@ -208,9 +208,6 @@
     <t>R</t>
   </si>
   <si>
-    <t>T-cells: CD4 CD8a</t>
-  </si>
-  <si>
     <t>Cells per condition in UMAPs etc.</t>
   </si>
   <si>
@@ -286,9 +283,6 @@
     <t>Control</t>
   </si>
   <si>
-    <t>NK and NK-Tcells: TCRb NK1.1</t>
-  </si>
-  <si>
     <t>Control over Treatment</t>
   </si>
   <si>
@@ -491,6 +485,30 @@
   </si>
   <si>
     <t>Choose whether to run QC, and if so, which method.</t>
+  </si>
+  <si>
+    <t>Bcells: CD19 MHC-II</t>
+  </si>
+  <si>
+    <t>DCs: CD11c MHC-II</t>
+  </si>
+  <si>
+    <t>Neutrophils: CD11b Ly6G</t>
+  </si>
+  <si>
+    <t>Macrophages: F4-80 CD11b</t>
+  </si>
+  <si>
+    <t>Eos: Siglec-F CD11b</t>
+  </si>
+  <si>
+    <t>CD4: TCRb CD4</t>
+  </si>
+  <si>
+    <t>NK-Tcells: TCRb NK1.1</t>
+  </si>
+  <si>
+    <t>NK Cells: NK1.1+ CD3-</t>
   </si>
 </sst>
 </file>
@@ -1001,10 +1019,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1326,220 +1340,220 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A1" s="6" t="s">
+        <v>98</v>
+      </c>
+      <c r="B1" s="10" t="s">
+        <v>99</v>
+      </c>
+      <c r="C1" s="5" t="s">
         <v>100</v>
-      </c>
-      <c r="B1" s="10" t="s">
-        <v>101</v>
-      </c>
-      <c r="C1" s="5" t="s">
-        <v>102</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A2" s="11" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="B2" s="12">
         <v>1000</v>
       </c>
       <c r="C2" s="13" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A3" s="14" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="B3" s="15" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="C3" s="16" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A4" s="14" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="B4" s="15" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="C4" s="16" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A5" s="14" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="B5" s="15" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="C5" s="16" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A6" s="14" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="B6" s="15">
         <v>20</v>
       </c>
       <c r="C6" s="16" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A7" s="17" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="B7" s="18" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="C7" s="19" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A8" s="17" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="B8" s="18" t="s">
         <v>47</v>
       </c>
       <c r="C8" s="19" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A9" s="20" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="B9" s="21" t="s">
+        <v>143</v>
+      </c>
+      <c r="C9" s="22" t="s">
         <v>145</v>
-      </c>
-      <c r="C9" s="22" t="s">
-        <v>147</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A10" s="20" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="B10" s="21" t="b">
         <v>0</v>
       </c>
       <c r="C10" s="22" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A11" s="23" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="B11" s="24"/>
       <c r="C11" s="25" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A12" s="23" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="B12" s="24" t="b">
         <v>0</v>
       </c>
       <c r="C12" s="25" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A13" s="23" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="B13" s="24" t="b">
         <v>0</v>
       </c>
       <c r="C13" s="25" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A14" s="23" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="B14" s="24" t="b">
         <v>1</v>
       </c>
       <c r="C14" s="25" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A15" s="23" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="B15" s="24">
         <v>4</v>
       </c>
       <c r="C15" s="25" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A16" s="23" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="B16" s="24">
         <v>6</v>
       </c>
       <c r="C16" s="25" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A17" s="23" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="B17" s="24" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="C17" s="25" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A18" s="23" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="B18" s="24" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="C18" s="25" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A19" s="26" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="B19" s="27" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="C19" s="28" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A20" s="29" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="B20" s="30" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="C20" s="31" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.2">
@@ -1651,7 +1665,7 @@
         <v>16</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C1" s="4" t="s">
         <v>0</v>
@@ -1674,13 +1688,13 @@
     </row>
     <row r="2" spans="1:8" ht="19" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>77</v>
+      </c>
+      <c r="B2" t="s">
+        <v>54</v>
+      </c>
+      <c r="C2" t="s">
         <v>78</v>
-      </c>
-      <c r="B2" t="s">
-        <v>55</v>
-      </c>
-      <c r="C2" t="s">
-        <v>80</v>
       </c>
       <c r="D2" t="s">
         <v>13</v>
@@ -1700,13 +1714,13 @@
     </row>
     <row r="3" spans="1:8" ht="19" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B3" t="s">
+        <v>55</v>
+      </c>
+      <c r="D3" t="s">
         <v>56</v>
-      </c>
-      <c r="D3" t="s">
-        <v>57</v>
       </c>
       <c r="E3" t="s">
         <v>47</v>
@@ -1718,7 +1732,7 @@
         <v>7</v>
       </c>
       <c r="H3" t="s">
-        <v>53</v>
+        <v>151</v>
       </c>
     </row>
     <row r="4" spans="1:8" ht="19" x14ac:dyDescent="0.25">
@@ -1735,7 +1749,7 @@
         <v>6</v>
       </c>
       <c r="H4" t="s">
-        <v>79</v>
+        <v>152</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="19" x14ac:dyDescent="0.25">
@@ -1751,6 +1765,9 @@
       <c r="G5" t="s">
         <v>5</v>
       </c>
+      <c r="H5" t="s">
+        <v>146</v>
+      </c>
     </row>
     <row r="6" spans="1:8" ht="19" x14ac:dyDescent="0.25">
       <c r="D6" t="s">
@@ -1765,6 +1782,9 @@
       <c r="G6" t="s">
         <v>4</v>
       </c>
+      <c r="H6" t="s">
+        <v>147</v>
+      </c>
     </row>
     <row r="7" spans="1:8" ht="19" x14ac:dyDescent="0.25">
       <c r="D7" t="s">
@@ -1779,10 +1799,13 @@
       <c r="G7" t="s">
         <v>17</v>
       </c>
+      <c r="H7" t="s">
+        <v>148</v>
+      </c>
     </row>
     <row r="8" spans="1:8" ht="19" x14ac:dyDescent="0.25">
       <c r="D8" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="E8" t="s">
         <v>47</v>
@@ -1793,10 +1816,13 @@
       <c r="G8" t="s">
         <v>18</v>
       </c>
+      <c r="H8" t="s">
+        <v>149</v>
+      </c>
     </row>
     <row r="9" spans="1:8" ht="19" x14ac:dyDescent="0.25">
       <c r="D9" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="E9" t="s">
         <v>47</v>
@@ -1806,6 +1832,9 @@
       </c>
       <c r="G9" t="s">
         <v>9</v>
+      </c>
+      <c r="H9" t="s">
+        <v>150</v>
       </c>
     </row>
     <row r="10" spans="1:8" ht="19" x14ac:dyDescent="0.25">
@@ -1821,6 +1850,9 @@
       <c r="G10" t="s">
         <v>10</v>
       </c>
+      <c r="H10" t="s">
+        <v>153</v>
+      </c>
     </row>
     <row r="11" spans="1:8" ht="19" x14ac:dyDescent="0.25">
       <c r="D11" t="s">
@@ -1833,7 +1865,7 @@
         <v>2500</v>
       </c>
       <c r="G11" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="12" spans="1:8" ht="19" x14ac:dyDescent="0.25">
@@ -1847,7 +1879,7 @@
         <v>2500</v>
       </c>
       <c r="G12" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="13" spans="1:8" ht="19" x14ac:dyDescent="0.25">
@@ -1907,7 +1939,7 @@
     </row>
     <row r="18" spans="4:6" ht="19" x14ac:dyDescent="0.25">
       <c r="D18" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="E18" t="s">
         <v>48</v>
@@ -1918,7 +1950,7 @@
     </row>
     <row r="19" spans="4:6" ht="19" x14ac:dyDescent="0.25">
       <c r="D19" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E19" t="s">
         <v>48</v>
@@ -1951,7 +1983,7 @@
     </row>
     <row r="22" spans="4:6" ht="19" x14ac:dyDescent="0.25">
       <c r="D22" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="E22" t="s">
         <v>48</v>
@@ -1962,7 +1994,7 @@
     </row>
     <row r="23" spans="4:6" ht="19" x14ac:dyDescent="0.25">
       <c r="D23" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="E23" t="s">
         <v>47</v>
@@ -2024,13 +2056,13 @@
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B2" t="s">
         <v>49</v>
       </c>
       <c r="C2" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="D2" t="s">
         <v>51</v>
@@ -2038,13 +2070,13 @@
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B3" t="s">
         <v>26</v>
       </c>
       <c r="C3" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="D3" t="s">
         <v>52</v>
@@ -2052,13 +2084,13 @@
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B4" t="s">
         <v>27</v>
       </c>
       <c r="C4" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="D4" t="s">
         <v>51</v>
@@ -2066,13 +2098,13 @@
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B5" t="s">
         <v>28</v>
       </c>
       <c r="C5" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="D5" t="s">
         <v>52</v>
@@ -2080,13 +2112,13 @@
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B6" t="s">
         <v>29</v>
       </c>
       <c r="C6" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="D6" t="s">
         <v>51</v>
@@ -2094,13 +2126,13 @@
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B7" t="s">
         <v>30</v>
       </c>
       <c r="C7" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="D7" t="s">
         <v>52</v>
@@ -2108,13 +2140,13 @@
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B8" t="s">
         <v>31</v>
       </c>
       <c r="C8" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D8" t="s">
         <v>51</v>
@@ -2122,13 +2154,13 @@
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B9" t="s">
         <v>32</v>
       </c>
       <c r="C9" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D9" t="s">
         <v>52</v>
@@ -2136,13 +2168,13 @@
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B10" t="s">
         <v>33</v>
       </c>
       <c r="C10" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D10" t="s">
         <v>51</v>
@@ -2150,13 +2182,13 @@
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B11" t="s">
         <v>34</v>
       </c>
       <c r="C11" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D11" t="s">
         <v>51</v>
@@ -2164,13 +2196,13 @@
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B12" t="s">
         <v>35</v>
       </c>
       <c r="C12" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D12" t="s">
         <v>52</v>
@@ -2192,22 +2224,22 @@
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="B1" t="s">
         <v>47</v>
       </c>
       <c r="C1" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="D1" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="E1" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="F1" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="G1" t="b">
         <v>1</v>
@@ -2215,22 +2247,22 @@
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="B2" t="s">
         <v>48</v>
       </c>
       <c r="C2" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="D2" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="E2" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="F2" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="G2" t="b">
         <v>0</v>
@@ -2238,56 +2270,56 @@
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="B3" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="C3" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="D3" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="E3" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="F3" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="E4" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="F4" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.2">
       <c r="E5" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="F5" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.2">
       <c r="F6" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.2">
       <c r="F7" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.2">
       <c r="F8" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add bundled MfastPG + Mphenograph, replace FastPG, make Rphenograph optional
Pure R PhenoGraph implementations that always install from CRAN deps:
- Mphenograph: exact k-NN (RANN) + Jaccard + Louvain
- MfastPG: approximate k-NN (RcppHNSW) + Jaccard + Louvain, ~10-17x faster

Updates across pipeline, Shiny app, Tauri GUI, install flow, and tests.
Moves Nebulosa from Imports to Suggests.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/inst/pipeline/MARMOT_Metadata.xlsx
+++ b/inst/pipeline/MARMOT_Metadata.xlsx
@@ -1,18 +1,25 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10222"/>
   <workbookPr defaultThemeVersion="166925"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/peterleary/Desktop/marmot/inst/pipeline/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A68404DC-9563-5B43-9B38-B62407FA469A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="15660" yWindow="4620" windowWidth="34560" windowHeight="20440" firstSheet="0" activeTab="1"/>
+    <workbookView xWindow="6560" yWindow="4620" windowWidth="34560" windowHeight="20440" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Pipeline Settings" sheetId="3" state="visible" r:id="rId1"/>
-    <sheet name="Study Data" sheetId="1" state="visible" r:id="rId2"/>
-    <sheet name="File Data" sheetId="2" state="visible" r:id="rId3"/>
+    <sheet name="Pipeline Settings" sheetId="3" r:id="rId1"/>
+    <sheet name="Study Data" sheetId="1" r:id="rId2"/>
+    <sheet name="File Data" sheetId="2" r:id="rId3"/>
     <sheet name="Options" sheetId="4" state="hidden" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="clusteringMethodToUse" localSheetId="3">Options!$A$1:$A$4</definedName>
+    <definedName name="clusteringMethodToUse" localSheetId="3">Options!$A$1:$A$5</definedName>
     <definedName name="dimRedMethodToUse">Options!$C$1:$C$3</definedName>
     <definedName name="markersToClusterBy">Options!$B$1:$B$3</definedName>
     <definedName name="qcDropdown">Options!$D$1:$D$3</definedName>
@@ -20,12 +27,12 @@
     <definedName name="themeToUse">Options!$E$1:$E$5</definedName>
     <definedName name="viridisColour">Options!$F$1:$F$8</definedName>
   </definedNames>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="208" uniqueCount="208">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="218" uniqueCount="170">
   <si>
     <t>Conditions To Test</t>
   </si>
@@ -264,400 +271,293 @@
     <t>Control over Treatment</t>
   </si>
   <si>
+    <t>FlowSOM</t>
+  </si>
+  <si>
+    <t>Rphenograph</t>
+  </si>
+  <si>
+    <t>PARC</t>
+  </si>
+  <si>
+    <t>all</t>
+  </si>
+  <si>
+    <t>UMAP</t>
+  </si>
+  <si>
+    <t>TSNE</t>
+  </si>
+  <si>
+    <t>pacmap</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Click on the available DR methods to use. If selecting pacmap, please make sure it is installed correctly first. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Do you want to save lots of the figures as PDFs? </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Enter the number of processor cores the pipeline can use. Don’t use all! </t>
+  </si>
+  <si>
+    <t>prism</t>
+  </si>
+  <si>
+    <t>classic</t>
+  </si>
+  <si>
+    <t>bw</t>
+  </si>
+  <si>
+    <t>minimal</t>
+  </si>
+  <si>
+    <t>void</t>
+  </si>
+  <si>
+    <t>viridis</t>
+  </si>
+  <si>
+    <t>magma</t>
+  </si>
+  <si>
+    <t>plasma</t>
+  </si>
+  <si>
+    <t>inferno</t>
+  </si>
+  <si>
+    <t>cividis</t>
+  </si>
+  <si>
+    <t>mako</t>
+  </si>
+  <si>
+    <t>rocket</t>
+  </si>
+  <si>
+    <t>turbo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Select a viridis theme to use. Marmots like mako. </t>
+  </si>
+  <si>
+    <t>None</t>
+  </si>
+  <si>
+    <t>PeacoQC</t>
+  </si>
+  <si>
+    <t>FlowAI</t>
+  </si>
+  <si>
+    <t>Bcells: CD19 MHC-II</t>
+  </si>
+  <si>
+    <t>DCs: CD11c MHC-II</t>
+  </si>
+  <si>
+    <t>Neutrophils: CD11b Ly6G</t>
+  </si>
+  <si>
+    <t>Macrophages: F4-80 CD11b</t>
+  </si>
+  <si>
+    <t>Eos: Siglec-F CD11b</t>
+  </si>
+  <si>
+    <t>CD4: TCRb CD4</t>
+  </si>
+  <si>
+    <t>NK-Tcells: TCRb NK1.1</t>
+  </si>
+  <si>
+    <t>NK Cells: NK1.1+ CD3-</t>
+  </si>
+  <si>
+    <t>Variable</t>
+  </si>
+  <si>
+    <t>Setting</t>
+  </si>
+  <si>
+    <t>Info</t>
+  </si>
+  <si>
+    <t>downsampleTo</t>
+  </si>
+  <si>
+    <t>1000</t>
+  </si>
+  <si>
+    <t>Number of cells to take from each FCS file. Leave blank to include all cells (will make things slow).</t>
+  </si>
+  <si>
+    <t>clusteringMethodToUse</t>
+  </si>
+  <si>
+    <t>FlowSOM</t>
+  </si>
+  <si>
+    <t>Click one of the available clustering methods to use. FlowSOM comes as default. The others, you will need to ensure that you installed them correctly.</t>
+  </si>
+  <si>
+    <t>markersToClusterBy</t>
+  </si>
+  <si>
+    <t>all</t>
+  </si>
+  <si>
+    <t>Click one of the available marker types to use. If you only have, say, state markers, select either all or state.</t>
+  </si>
+  <si>
+    <t>kValuesIWant</t>
+  </si>
+  <si>
+    <t>20 40 60</t>
+  </si>
+  <si>
+    <t>Number of knn/metacluster values to include in some of the visualisation, to see how over-/under-clustered you are. Space separated numbers, please.</t>
+  </si>
+  <si>
+    <t>knn</t>
+  </si>
+  <si>
+    <t>20</t>
+  </si>
+  <si>
+    <t>The actual knn/metacluster value to use for the main results, including differential abundance</t>
+  </si>
+  <si>
+    <t>dimRedMethodToUse</t>
+  </si>
+  <si>
+    <t>UMAP</t>
+  </si>
+  <si>
+    <t>markersToDimRedBy</t>
+  </si>
+  <si>
+    <t>type</t>
+  </si>
+  <si>
+    <t>runQC</t>
+  </si>
+  <si>
+    <t>PeacoQC</t>
+  </si>
+  <si>
+    <t>Choose whether to run QC, and if so, which method.</t>
+  </si>
+  <si>
+    <t>useQC</t>
+  </si>
+  <si>
+    <t>FALSE</t>
+  </si>
+  <si>
+    <t>Choose whether to use the QC-cleaned FCS files.</t>
+  </si>
+  <si>
+    <t>RDataFolder</t>
+  </si>
+  <si>
+    <t>If you ran marmot already and want to load in those results, paste in the filepath here. Leave blank otherwise.</t>
+  </si>
+  <si>
+    <t>gimmePDFs</t>
+  </si>
+  <si>
+    <t>quantileNormaliseAll</t>
+  </si>
+  <si>
+    <t>Do you want to use the 99% quantile normalised counts for all the analyses, including clustering and DR? Select FALSE if not sure.</t>
+  </si>
+  <si>
+    <t>runInParallel</t>
+  </si>
+  <si>
+    <t>TRUE</t>
+  </si>
+  <si>
+    <t>Try and speed things up a bit? Select TRUE.</t>
+  </si>
+  <si>
+    <t>nCores</t>
+  </si>
+  <si>
+    <t>4</t>
+  </si>
+  <si>
+    <t>ramPerCore</t>
+  </si>
+  <si>
+    <t>6</t>
+  </si>
+  <si>
+    <t>Enter an amount of RAM per processor core. Marmot likes at least 6. Make sure nCores*ramPerCore is less than your total amount of RAM</t>
+  </si>
+  <si>
+    <t>themeToUse</t>
+  </si>
+  <si>
+    <t>prism</t>
+  </si>
+  <si>
+    <t>Select a ggplot theme to use. Marmots like prism.</t>
+  </si>
+  <si>
+    <t>viridisColour</t>
+  </si>
+  <si>
+    <t>mako</t>
+  </si>
+  <si>
     <t>condaDir</t>
   </si>
   <si>
+    <t>~/miniforge3/bin/mamba</t>
+  </si>
+  <si>
+    <t>If you selected PARC and/or PacMAP, tell me where conda/mamba lives. Leave blank otherwise.</t>
+  </si>
+  <si>
     <t>parcScriptDir</t>
   </si>
   <si>
-    <t>downsampleTo</t>
-  </si>
-  <si>
-    <t>clusteringMethodToUse</t>
-  </si>
-  <si>
-    <t>markersToClusterBy</t>
-  </si>
-  <si>
-    <t>kValuesIWant</t>
-  </si>
-  <si>
-    <t>knn</t>
-  </si>
-  <si>
-    <t>dimRedMethodToUse</t>
-  </si>
-  <si>
-    <t>markersToDimRedBy</t>
-  </si>
-  <si>
-    <t>runQC</t>
-  </si>
-  <si>
-    <t>useQC</t>
-  </si>
-  <si>
-    <t>RDataFolder</t>
-  </si>
-  <si>
-    <t>gimmePDFs</t>
-  </si>
-  <si>
-    <t>quantileNormaliseAll</t>
-  </si>
-  <si>
-    <t>runInParallel</t>
-  </si>
-  <si>
-    <t>nCores</t>
-  </si>
-  <si>
-    <t>ramPerCore</t>
-  </si>
-  <si>
-    <t>themeToUse</t>
-  </si>
-  <si>
-    <t>viridisColour</t>
-  </si>
-  <si>
-    <t>Variable</t>
-  </si>
-  <si>
-    <t>Setting</t>
-  </si>
-  <si>
-    <t>Info</t>
-  </si>
-  <si>
-    <t>FlowSOM</t>
-  </si>
-  <si>
-    <t>Rphenograph</t>
-  </si>
-  <si>
-    <t>PARC</t>
-  </si>
-  <si>
-    <t>FastPG</t>
-  </si>
-  <si>
-    <t>Click one of the available clustering methods to use. FlowSOM comes as default. The others, you will need to ensure that you installed them correctly.</t>
-  </si>
-  <si>
-    <t>all</t>
-  </si>
-  <si>
-    <t>Number of knn/metacluster values to include in some of the visualisation, to see how over-/under-clustered you are. Space separated numbers, please.</t>
-  </si>
-  <si>
-    <t>The actual knn/metacluster value to use for the main results, including differential abundance</t>
-  </si>
-  <si>
-    <t>UMAP</t>
-  </si>
-  <si>
-    <t>TSNE</t>
-  </si>
-  <si>
-    <t>pacmap</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Click on the available DR methods to use. If selecting pacmap, please make sure it is installed correctly first. </t>
-  </si>
-  <si>
-    <t>Click one of the available marker types to use. If you only have, say, state markers, select either all or state.</t>
-  </si>
-  <si>
-    <t>Choose whether to use the QC-cleaned FCS files.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Do you want to save lots of the figures as PDFs? </t>
-  </si>
-  <si>
-    <t>Do you want to use the 99% quantile normalised counts for all the analyses, including clustering and DR? Select FALSE if not sure.</t>
-  </si>
-  <si>
-    <t>Try and speed things up a bit? Select TRUE.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Enter the number of processor cores the pipeline can use. Don’t use all! </t>
-  </si>
-  <si>
-    <t>prism</t>
-  </si>
-  <si>
-    <t>classic</t>
-  </si>
-  <si>
-    <t>bw</t>
-  </si>
-  <si>
-    <t>minimal</t>
-  </si>
-  <si>
-    <t>void</t>
-  </si>
-  <si>
-    <t>viridis</t>
-  </si>
-  <si>
-    <t>magma</t>
-  </si>
-  <si>
-    <t>plasma</t>
-  </si>
-  <si>
-    <t>inferno</t>
-  </si>
-  <si>
-    <t>cividis</t>
-  </si>
-  <si>
-    <t>mako</t>
-  </si>
-  <si>
-    <t>rocket</t>
-  </si>
-  <si>
-    <t>turbo</t>
-  </si>
-  <si>
-    <t>20 40 60</t>
-  </si>
-  <si>
-    <t>If you ran marmot already and want to load in those results, paste in the filepath here. Leave blank otherwise.</t>
-  </si>
-  <si>
-    <t>~/miniforge3/bin/mamba</t>
-  </si>
-  <si>
-    <t>If you selected PARC and/or PacMAP, tell me where conda/mamba lives. Leave blank otherwise.</t>
+    <t>~/Desktop/MARMOT/</t>
   </si>
   <si>
     <t>Tell me where you saved Stephan Benke-Bruderer's PARC and PacMAP script. Leave blank otherwise.</t>
   </si>
   <si>
-    <t>~/Desktop/MARMOT/</t>
-  </si>
-  <si>
-    <t>Number of cells to take from each FCS file. Leave blank to include all cells (will make things slow).</t>
-  </si>
-  <si>
-    <t>Enter an amount of RAM per processor core. Marmot likes at least 6. Make sure nCores*ramPerCore is less than your total amount of RAM</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Select a viridis theme to use. Marmots like mako. </t>
-  </si>
-  <si>
-    <t>Select a ggplot theme to use. Marmots like prism.</t>
-  </si>
-  <si>
-    <t>None</t>
-  </si>
-  <si>
-    <t>PeacoQC</t>
-  </si>
-  <si>
-    <t>FlowAI</t>
-  </si>
-  <si>
-    <t>Choose whether to run QC, and if so, which method.</t>
-  </si>
-  <si>
-    <t>Bcells: CD19 MHC-II</t>
-  </si>
-  <si>
-    <t>DCs: CD11c MHC-II</t>
-  </si>
-  <si>
-    <t>Neutrophils: CD11b Ly6G</t>
-  </si>
-  <si>
-    <t>Macrophages: F4-80 CD11b</t>
-  </si>
-  <si>
-    <t>Eos: Siglec-F CD11b</t>
-  </si>
-  <si>
-    <t>CD4: TCRb CD4</t>
-  </si>
-  <si>
-    <t>NK-Tcells: TCRb NK1.1</t>
-  </si>
-  <si>
-    <t>NK Cells: NK1.1+ CD3-</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Variable</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Setting</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Info</t>
-  </si>
-  <si>
-    <t xml:space="preserve">downsampleTo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1000</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Number of cells to take from each FCS file. Leave blank to include all cells (will make things slow).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">clusteringMethodToUse</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FlowSOM</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Click one of the available clustering methods to use. FlowSOM comes as default. The others, you will need to ensure that you installed them correctly.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">markersToClusterBy</t>
-  </si>
-  <si>
-    <t xml:space="preserve">all</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Click one of the available marker types to use. If you only have, say, state markers, select either all or state.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">kValuesIWant</t>
-  </si>
-  <si>
-    <t xml:space="preserve">20 40 60</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Number of knn/metacluster values to include in some of the visualisation, to see how over-/under-clustered you are. Space separated numbers, please.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">knn</t>
-  </si>
-  <si>
-    <t xml:space="preserve">20</t>
-  </si>
-  <si>
-    <t xml:space="preserve">The actual knn/metacluster value to use for the main results, including differential abundance</t>
-  </si>
-  <si>
-    <t xml:space="preserve">dimRedMethodToUse</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UMAP</t>
-  </si>
-  <si>
-    <t xml:space="preserve">markersToDimRedBy</t>
-  </si>
-  <si>
-    <t xml:space="preserve">type</t>
-  </si>
-  <si>
-    <t xml:space="preserve">runQC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PeacoQC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Choose whether to run QC, and if so, which method.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">useQC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FALSE</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Choose whether to use the QC-cleaned FCS files.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">RDataFolder</t>
-  </si>
-  <si>
-    <t xml:space="preserve">If you ran marmot already and want to load in those results, paste in the filepath here. Leave blank otherwise.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">gimmePDFs</t>
-  </si>
-  <si>
-    <t xml:space="preserve">quantileNormaliseAll</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Do you want to use the 99% quantile normalised counts for all the analyses, including clustering and DR? Select FALSE if not sure.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">runInParallel</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TRUE</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Try and speed things up a bit? Select TRUE.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">nCores</t>
-  </si>
-  <si>
-    <t xml:space="preserve">4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ramPerCore</t>
-  </si>
-  <si>
-    <t xml:space="preserve">6</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Enter an amount of RAM per processor core. Marmot likes at least 6. Make sure nCores*ramPerCore is less than your total amount of RAM</t>
-  </si>
-  <si>
-    <t xml:space="preserve">themeToUse</t>
-  </si>
-  <si>
-    <t xml:space="preserve">prism</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Select a ggplot theme to use. Marmots like prism.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">viridisColour</t>
-  </si>
-  <si>
-    <t xml:space="preserve">mako</t>
-  </si>
-  <si>
-    <t xml:space="preserve">condaDir</t>
-  </si>
-  <si>
-    <t xml:space="preserve">~/miniforge3/bin/mamba</t>
-  </si>
-  <si>
-    <t xml:space="preserve">If you selected PARC and/or PacMAP, tell me where conda/mamba lives. Leave blank otherwise.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">parcScriptDir</t>
-  </si>
-  <si>
-    <t xml:space="preserve">~/Desktop/MARMOT/</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tell me where you saved Stephan Benke-Bruderer's PARC and PacMAP script. Leave blank otherwise.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">runScGate</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Run scGate marker-pair gating? Requires scGate, UCell, and Seurat. Fill in Marker Pairs in Study Data.</t>
+    <t>runScGate</t>
+  </si>
+  <si>
+    <t>Run scGate marker-pair gating? Requires scGate, UCell, and Seurat. Fill in Marker Pairs in Study Data.</t>
+  </si>
+  <si>
+    <t>Mphenograph</t>
+  </si>
+  <si>
+    <t>MfastPG</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="0"/>
-  <fonts count="5">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="12"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -669,13 +569,6 @@
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <scheme val="minor"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
     </font>
     <font>
       <sz val="14"/>
@@ -685,12 +578,12 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <b/>
       <sz val="22"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-      <b/>
     </font>
   </fonts>
   <fills count="9">
@@ -758,11 +651,14 @@
       <right style="thin">
         <color indexed="64"/>
       </right>
+      <top/>
       <bottom style="thin">
         <color indexed="64"/>
       </bottom>
+      <diagonal/>
     </border>
     <border>
+      <left/>
       <right style="thin">
         <color indexed="64"/>
       </right>
@@ -772,6 +668,7 @@
       <bottom style="thin">
         <color indexed="64"/>
       </bottom>
+      <diagonal/>
     </border>
     <border>
       <left style="thin">
@@ -786,25 +683,31 @@
       <bottom style="thin">
         <color indexed="64"/>
       </bottom>
+      <diagonal/>
     </border>
     <border>
       <left style="thin">
         <color indexed="64"/>
       </left>
+      <right/>
       <top style="thin">
         <color indexed="64"/>
       </top>
       <bottom style="thin">
         <color indexed="64"/>
       </bottom>
+      <diagonal/>
     </border>
     <border>
+      <left/>
       <right style="thin">
         <color indexed="64"/>
       </right>
       <top style="thin">
         <color indexed="64"/>
       </top>
+      <bottom/>
+      <diagonal/>
     </border>
     <border>
       <left style="thin">
@@ -816,35 +719,50 @@
       <top style="thin">
         <color indexed="64"/>
       </top>
+      <bottom/>
+      <diagonal/>
     </border>
     <border>
       <left style="thin">
         <color indexed="64"/>
       </left>
+      <right/>
       <top style="thin">
         <color indexed="64"/>
       </top>
+      <bottom/>
+      <diagonal/>
     </border>
     <border>
       <left style="thin">
         <color indexed="64"/>
       </left>
+      <right/>
+      <top/>
       <bottom style="thin">
         <color indexed="64"/>
       </bottom>
+      <diagonal/>
     </border>
     <border>
+      <left/>
       <right style="thin">
         <color indexed="64"/>
       </right>
+      <top/>
       <bottom style="thin">
         <color indexed="64"/>
       </bottom>
+      <diagonal/>
     </border>
     <border>
+      <left/>
+      <right/>
       <top style="thin">
         <color indexed="64"/>
       </top>
+      <bottom/>
+      <diagonal/>
     </border>
     <border>
       <left style="medium">
@@ -859,6 +777,7 @@
       <bottom style="medium">
         <color indexed="64"/>
       </bottom>
+      <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
@@ -938,7 +857,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="10">
+  <dxfs count="2">
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -958,166 +877,6 @@
           <bgColor rgb="FFFFC7CE"/>
         </patternFill>
       </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right/>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left/>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-      </border>
-    </dxf>
-    <dxf>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
-    <dxf>
-      <border>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top/>
-        <bottom/>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal style="thin">
-          <color indexed="64"/>
-        </horizontal>
-      </border>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -1428,242 +1187,242 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:C21"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="20.83203125" hidden="0" customWidth="1"/>
-    <col min="2" max="2" width="22.83203125" hidden="0" customWidth="1"/>
-    <col min="3" max="3" width="128.6640625" hidden="0" customWidth="1"/>
+    <col min="1" max="1" width="20.83203125" customWidth="1"/>
+    <col min="2" max="2" width="22.83203125" customWidth="1"/>
+    <col min="3" max="3" width="128.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A1" s="24" t="s">
-        <v>154</v>
+        <v>114</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>155</v>
+        <v>115</v>
       </c>
       <c r="C1" s="23" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="2">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
-        <v>157</v>
+        <v>117</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>158</v>
+        <v>118</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>159</v>
-      </c>
-    </row>
-    <row r="3">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A3" s="5" t="s">
-        <v>160</v>
+        <v>120</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>161</v>
+        <v>121</v>
       </c>
       <c r="C3" s="7" t="s">
-        <v>162</v>
-      </c>
-    </row>
-    <row r="4">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A4" s="5" t="s">
-        <v>163</v>
+        <v>123</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>164</v>
+        <v>124</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>165</v>
-      </c>
-    </row>
-    <row r="5">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A5" s="5" t="s">
-        <v>166</v>
+        <v>126</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>167</v>
+        <v>127</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="6">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A6" s="5" t="s">
-        <v>169</v>
+        <v>129</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>170</v>
+        <v>130</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>171</v>
-      </c>
-    </row>
-    <row r="7">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A7" s="8" t="s">
-        <v>172</v>
+        <v>132</v>
       </c>
       <c r="B7" s="9" t="s">
-        <v>173</v>
+        <v>133</v>
       </c>
       <c r="C7" s="10" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="8">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A8" s="8" t="s">
-        <v>174</v>
+        <v>134</v>
       </c>
       <c r="B8" s="9" t="s">
-        <v>175</v>
+        <v>135</v>
       </c>
       <c r="C8" s="10" t="s">
-        <v>165</v>
-      </c>
-    </row>
-    <row r="9">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A9" s="11" t="s">
-        <v>176</v>
+        <v>136</v>
       </c>
       <c r="B9" s="12" t="s">
-        <v>177</v>
+        <v>137</v>
       </c>
       <c r="C9" s="13" t="s">
-        <v>178</v>
-      </c>
-    </row>
-    <row r="10">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A10" s="11" t="s">
-        <v>179</v>
+        <v>139</v>
       </c>
       <c r="B10" s="12" t="s">
-        <v>180</v>
+        <v>140</v>
       </c>
       <c r="C10" s="13" t="s">
-        <v>181</v>
-      </c>
-    </row>
-    <row r="11">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A11" s="14" t="s">
-        <v>182</v>
+        <v>142</v>
       </c>
       <c r="B11" s="15"/>
       <c r="C11" s="16" t="s">
-        <v>183</v>
-      </c>
-    </row>
-    <row r="12">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A12" s="14" t="s">
-        <v>184</v>
+        <v>144</v>
       </c>
       <c r="B12" s="15" t="s">
-        <v>180</v>
+        <v>140</v>
       </c>
       <c r="C12" s="16" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="13">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A13" s="14" t="s">
-        <v>185</v>
+        <v>145</v>
       </c>
       <c r="B13" s="15" t="s">
-        <v>180</v>
+        <v>140</v>
       </c>
       <c r="C13" s="16" t="s">
-        <v>186</v>
-      </c>
-    </row>
-    <row r="14">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A14" s="14" t="s">
-        <v>187</v>
+        <v>147</v>
       </c>
       <c r="B14" s="15" t="s">
-        <v>188</v>
+        <v>148</v>
       </c>
       <c r="C14" s="16" t="s">
-        <v>189</v>
-      </c>
-    </row>
-    <row r="15">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A15" s="14" t="s">
-        <v>190</v>
+        <v>150</v>
       </c>
       <c r="B15" s="15" t="s">
-        <v>191</v>
+        <v>151</v>
       </c>
       <c r="C15" s="16" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="16">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A16" s="14" t="s">
-        <v>192</v>
+        <v>152</v>
       </c>
       <c r="B16" s="15" t="s">
-        <v>193</v>
+        <v>153</v>
       </c>
       <c r="C16" s="16" t="s">
-        <v>194</v>
-      </c>
-    </row>
-    <row r="17">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A17" s="14" t="s">
-        <v>195</v>
+        <v>155</v>
       </c>
       <c r="B17" s="15" t="s">
-        <v>196</v>
+        <v>156</v>
       </c>
       <c r="C17" s="16" t="s">
-        <v>197</v>
-      </c>
-    </row>
-    <row r="18">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A18" s="14" t="s">
-        <v>198</v>
+        <v>158</v>
       </c>
       <c r="B18" s="15" t="s">
-        <v>199</v>
+        <v>159</v>
       </c>
       <c r="C18" s="16" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A19" s="17" t="s">
+        <v>160</v>
+      </c>
+      <c r="B19" s="18" t="s">
+        <v>161</v>
+      </c>
+      <c r="C19" s="19" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A20" s="20" t="s">
+        <v>163</v>
+      </c>
+      <c r="B20" s="21" t="s">
+        <v>164</v>
+      </c>
+      <c r="C20" s="22" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A21" s="25" t="s">
+        <v>166</v>
+      </c>
+      <c r="B21" s="25" t="s">
         <v>140</v>
       </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="17" t="s">
-        <v>200</v>
-      </c>
-      <c r="B19" s="18" t="s">
-        <v>201</v>
-      </c>
-      <c r="C19" s="19" t="s">
-        <v>202</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="20" t="s">
-        <v>203</v>
-      </c>
-      <c r="B20" s="21" t="s">
-        <v>204</v>
-      </c>
-      <c r="C20" s="22" t="s">
-        <v>205</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="25" t="s">
-        <v>206</v>
-      </c>
-      <c r="B21" s="25" t="s">
-        <v>180</v>
-      </c>
       <c r="C21" s="26" t="s">
-        <v>207</v>
+        <v>167</v>
       </c>
     </row>
   </sheetData>
@@ -1673,7 +1432,7 @@
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
       <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="11">
@@ -1695,6 +1454,24 @@
           </x14:formula1>
           <xm:sqref>B10</xm:sqref>
         </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{EF0F4D8A-D969-2040-A7B2-4D843CC1D241}">
+          <x14:formula1>
+            <xm:f>Options!$E$1:$E$5</xm:f>
+          </x14:formula1>
+          <xm:sqref>B17</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{D6D0959A-58E3-6B40-9F0A-C50FD537F1F2}">
+          <x14:formula1>
+            <xm:f>Options!$F$1:$F$8</xm:f>
+          </x14:formula1>
+          <xm:sqref>B18</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{C81D77FB-D1A4-0B4C-B41A-E5791F351257}">
+          <x14:formula1>
+            <xm:f>Options!$D$1:$D$3</xm:f>
+          </x14:formula1>
+          <xm:sqref>B9</xm:sqref>
+        </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{EA79EA2F-903F-354F-BF4D-E09B45EA2C79}">
           <x14:formula1>
             <xm:f>Options!G1:G2</xm:f>
@@ -1713,27 +1490,9 @@
           </x14:formula1>
           <xm:sqref>B14</xm:sqref>
         </x14:dataValidation>
-        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{EF0F4D8A-D969-2040-A7B2-4D843CC1D241}">
-          <x14:formula1>
-            <xm:f>Options!$E$1:$E$5</xm:f>
-          </x14:formula1>
-          <xm:sqref>B17</xm:sqref>
-        </x14:dataValidation>
-        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{D6D0959A-58E3-6B40-9F0A-C50FD537F1F2}">
-          <x14:formula1>
-            <xm:f>Options!$F$1:$F$8</xm:f>
-          </x14:formula1>
-          <xm:sqref>B18</xm:sqref>
-        </x14:dataValidation>
-        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{C81D77FB-D1A4-0B4C-B41A-E5791F351257}">
-          <x14:formula1>
-            <xm:f>Options!$D$1:$D$3</xm:f>
-          </x14:formula1>
-          <xm:sqref>B9</xm:sqref>
-        </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{ED65EFD9-012C-8E42-BE3B-3B16546394D0}">
           <x14:formula1>
-            <xm:f>Options!A1:A4</xm:f>
+            <xm:f>Options!A1:A5</xm:f>
           </x14:formula1>
           <xm:sqref>B3</xm:sqref>
         </x14:dataValidation>
@@ -1750,21 +1509,19 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+  <dimension ref="A1:H25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="19.6640625" hidden="0" customWidth="1"/>
-    <col min="2" max="2" width="32.6640625" hidden="0" customWidth="1"/>
-    <col min="3" max="3" width="32.6640625" hidden="0" customWidth="1"/>
-    <col min="4" max="4" width="20.33203125" hidden="0" customWidth="1"/>
-    <col min="5" max="5" width="20.33203125" hidden="0" customWidth="1"/>
-    <col min="6" max="6" width="24.6640625" hidden="0" customWidth="1"/>
-    <col min="7" max="7" width="26.6640625" hidden="0" customWidth="1"/>
-    <col min="8" max="8" width="26" hidden="0" customWidth="1"/>
+    <col min="1" max="1" width="19.6640625" customWidth="1"/>
+    <col min="2" max="3" width="32.6640625" customWidth="1"/>
+    <col min="4" max="5" width="20.33203125" customWidth="1"/>
+    <col min="6" max="6" width="24.6640625" customWidth="1"/>
+    <col min="7" max="7" width="26.6640625" customWidth="1"/>
+    <col min="8" max="8" width="26" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="91" customHeight="1">
+    <row r="1" spans="1:8" ht="91" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="28" t="s">
         <v>16</v>
       </c>
@@ -1790,7 +1547,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="2" ht="19" customHeight="1">
+    <row r="2" spans="1:8" ht="19" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>77</v>
       </c>
@@ -1806,7 +1563,7 @@
       <c r="E2" t="s">
         <v>47</v>
       </c>
-      <c r="F2" s="27" t="n">
+      <c r="F2" s="27">
         <v>2500</v>
       </c>
       <c r="G2" t="s">
@@ -1816,7 +1573,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="3" ht="19" customHeight="1">
+    <row r="3" spans="1:8" ht="19" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>76</v>
       </c>
@@ -1829,323 +1586,323 @@
       <c r="E3" t="s">
         <v>47</v>
       </c>
-      <c r="F3" s="27" t="n">
+      <c r="F3" s="27">
         <v>2500</v>
       </c>
       <c r="G3" t="s">
         <v>7</v>
       </c>
       <c r="H3" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="4" ht="19" customHeight="1">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" ht="19" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D4" t="s">
         <v>41</v>
       </c>
       <c r="E4" t="s">
         <v>47</v>
       </c>
-      <c r="F4" s="27" t="n">
+      <c r="F4" s="27">
         <v>2500</v>
       </c>
       <c r="G4" t="s">
         <v>6</v>
       </c>
       <c r="H4" t="s">
-        <v>152</v>
-      </c>
-    </row>
-    <row r="5" ht="19" customHeight="1">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" ht="19" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D5" t="s">
         <v>36</v>
       </c>
       <c r="E5" t="s">
         <v>47</v>
       </c>
-      <c r="F5" s="27" t="n">
+      <c r="F5" s="27">
         <v>2500</v>
       </c>
       <c r="G5" t="s">
         <v>5</v>
       </c>
       <c r="H5" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="6" ht="19" customHeight="1">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" ht="19" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D6" t="s">
         <v>43</v>
       </c>
       <c r="E6" t="s">
         <v>47</v>
       </c>
-      <c r="F6" s="27" t="n">
+      <c r="F6" s="27">
         <v>2500</v>
       </c>
       <c r="G6" t="s">
         <v>4</v>
       </c>
       <c r="H6" t="s">
-        <v>147</v>
-      </c>
-    </row>
-    <row r="7" ht="19" customHeight="1">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" ht="19" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D7" t="s">
         <v>44</v>
       </c>
       <c r="E7" t="s">
         <v>47</v>
       </c>
-      <c r="F7" s="27" t="n">
+      <c r="F7" s="27">
         <v>2500</v>
       </c>
       <c r="G7" t="s">
         <v>17</v>
       </c>
       <c r="H7" t="s">
-        <v>148</v>
-      </c>
-    </row>
-    <row r="8" ht="19" customHeight="1">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" ht="19" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D8" t="s">
         <v>57</v>
       </c>
       <c r="E8" t="s">
         <v>47</v>
       </c>
-      <c r="F8" s="27" t="n">
+      <c r="F8" s="27">
         <v>2500</v>
       </c>
       <c r="G8" t="s">
         <v>18</v>
       </c>
       <c r="H8" t="s">
-        <v>149</v>
-      </c>
-    </row>
-    <row r="9" ht="19" customHeight="1">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" ht="19" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D9" t="s">
         <v>58</v>
       </c>
       <c r="E9" t="s">
         <v>47</v>
       </c>
-      <c r="F9" s="27" t="n">
+      <c r="F9" s="27">
         <v>2500</v>
       </c>
       <c r="G9" t="s">
         <v>9</v>
       </c>
       <c r="H9" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="10" ht="19" customHeight="1">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" ht="19" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D10" t="s">
         <v>38</v>
       </c>
       <c r="E10" t="s">
         <v>48</v>
       </c>
-      <c r="F10" s="27" t="n">
+      <c r="F10" s="27">
         <v>2500</v>
       </c>
       <c r="G10" t="s">
         <v>10</v>
       </c>
       <c r="H10" t="s">
-        <v>153</v>
-      </c>
-    </row>
-    <row r="11" ht="19" customHeight="1">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" ht="19" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D11" t="s">
         <v>37</v>
       </c>
       <c r="E11" t="s">
         <v>48</v>
       </c>
-      <c r="F11" s="27" t="n">
+      <c r="F11" s="27">
         <v>2500</v>
       </c>
       <c r="G11" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="12" ht="19" customHeight="1">
+    <row r="12" spans="1:8" ht="19" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D12" t="s">
         <v>24</v>
       </c>
       <c r="E12" t="s">
         <v>47</v>
       </c>
-      <c r="F12" s="27" t="n">
+      <c r="F12" s="27">
         <v>2500</v>
       </c>
       <c r="G12" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="13" ht="19" customHeight="1">
+    <row r="13" spans="1:8" ht="19" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D13" t="s">
         <v>39</v>
       </c>
       <c r="E13" t="s">
         <v>47</v>
       </c>
-      <c r="F13" s="27" t="n">
-        <v>2500</v>
-      </c>
-    </row>
-    <row r="14" ht="19" customHeight="1">
+      <c r="F13" s="27">
+        <v>2500</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" ht="19" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D14" t="s">
         <v>42</v>
       </c>
       <c r="E14" t="s">
         <v>47</v>
       </c>
-      <c r="F14" s="27" t="n">
-        <v>2500</v>
-      </c>
-    </row>
-    <row r="15" ht="19" customHeight="1">
+      <c r="F14" s="27">
+        <v>2500</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" ht="19" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D15" t="s">
         <v>14</v>
       </c>
       <c r="E15" t="s">
         <v>47</v>
       </c>
-      <c r="F15" s="27" t="n">
-        <v>2500</v>
-      </c>
-    </row>
-    <row r="16" ht="19" customHeight="1">
+      <c r="F15" s="27">
+        <v>2500</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" ht="19" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D16" t="s">
         <v>15</v>
       </c>
       <c r="E16" t="s">
         <v>47</v>
       </c>
-      <c r="F16" s="27" t="n">
-        <v>2500</v>
-      </c>
-    </row>
-    <row r="17" ht="19" customHeight="1">
+      <c r="F16" s="27">
+        <v>2500</v>
+      </c>
+    </row>
+    <row r="17" spans="4:6" ht="19" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D17" t="s">
         <v>45</v>
       </c>
       <c r="E17" t="s">
         <v>48</v>
       </c>
-      <c r="F17" s="27" t="n">
-        <v>2500</v>
-      </c>
-    </row>
-    <row r="18" ht="19" customHeight="1">
+      <c r="F17" s="27">
+        <v>2500</v>
+      </c>
+    </row>
+    <row r="18" spans="4:6" ht="19" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D18" t="s">
         <v>60</v>
       </c>
       <c r="E18" t="s">
         <v>48</v>
       </c>
-      <c r="F18" s="27" t="n">
-        <v>2500</v>
-      </c>
-    </row>
-    <row r="19" ht="19" customHeight="1">
+      <c r="F18" s="27">
+        <v>2500</v>
+      </c>
+    </row>
+    <row r="19" spans="4:6" ht="19" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D19" t="s">
         <v>61</v>
       </c>
       <c r="E19" t="s">
         <v>48</v>
       </c>
-      <c r="F19" s="27" t="n">
-        <v>2500</v>
-      </c>
-    </row>
-    <row r="20" ht="19" customHeight="1">
+      <c r="F19" s="27">
+        <v>2500</v>
+      </c>
+    </row>
+    <row r="20" spans="4:6" ht="19" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D20" t="s">
         <v>40</v>
       </c>
       <c r="E20" t="s">
         <v>48</v>
       </c>
-      <c r="F20" s="27" t="n">
-        <v>2500</v>
-      </c>
-    </row>
-    <row r="21" ht="19" customHeight="1">
+      <c r="F20" s="27">
+        <v>2500</v>
+      </c>
+    </row>
+    <row r="21" spans="4:6" ht="19" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D21" t="s">
         <v>19</v>
       </c>
       <c r="E21" t="s">
         <v>48</v>
       </c>
-      <c r="F21" s="27" t="n">
-        <v>2500</v>
-      </c>
-    </row>
-    <row r="22" ht="19" customHeight="1">
+      <c r="F21" s="27">
+        <v>2500</v>
+      </c>
+    </row>
+    <row r="22" spans="4:6" ht="19" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D22" t="s">
         <v>63</v>
       </c>
       <c r="E22" t="s">
         <v>48</v>
       </c>
-      <c r="F22" s="27" t="n">
-        <v>2500</v>
-      </c>
-    </row>
-    <row r="23" ht="19" customHeight="1">
+      <c r="F22" s="27">
+        <v>2500</v>
+      </c>
+    </row>
+    <row r="23" spans="4:6" ht="19" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D23" t="s">
         <v>64</v>
       </c>
       <c r="E23" t="s">
         <v>47</v>
       </c>
-      <c r="F23" s="27" t="n">
-        <v>2500</v>
-      </c>
-    </row>
-    <row r="24" ht="19" customHeight="1">
+      <c r="F23" s="27">
+        <v>2500</v>
+      </c>
+    </row>
+    <row r="24" spans="4:6" ht="19" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D24" t="s">
         <v>25</v>
       </c>
       <c r="E24" t="s">
         <v>48</v>
       </c>
-      <c r="F24" s="27" t="n">
-        <v>2500</v>
-      </c>
-    </row>
-    <row r="25" ht="19" customHeight="1">
+      <c r="F24" s="27">
+        <v>2500</v>
+      </c>
+    </row>
+    <row r="25" spans="4:6" ht="19" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D25" t="s">
         <v>46</v>
       </c>
       <c r="E25" t="s">
         <v>48</v>
       </c>
-      <c r="F25" s="27" t="n">
+      <c r="F25" s="27">
         <v>2500</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+  <dimension ref="A1:D12"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="72.5" hidden="0" customWidth="1"/>
-    <col min="2" max="2" width="18" hidden="0" customWidth="1"/>
-    <col min="3" max="3" width="19.6640625" hidden="0" customWidth="1"/>
+    <col min="1" max="1" width="72.5" customWidth="1"/>
+    <col min="2" max="2" width="18" customWidth="1"/>
+    <col min="3" max="3" width="19.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A1" s="29" t="s">
         <v>11</v>
       </c>
@@ -2159,7 +1916,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>65</v>
       </c>
@@ -2173,7 +1930,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="3">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>66</v>
       </c>
@@ -2187,7 +1944,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="4">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>67</v>
       </c>
@@ -2201,7 +1958,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="5">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>68</v>
       </c>
@@ -2215,7 +1972,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="6">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>69</v>
       </c>
@@ -2229,7 +1986,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="7">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>70</v>
       </c>
@@ -2243,7 +2000,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="8">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>71</v>
       </c>
@@ -2257,7 +2014,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="9">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>72</v>
       </c>
@@ -2271,7 +2028,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="10">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>73</v>
       </c>
@@ -2285,7 +2042,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="11">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>74</v>
       </c>
@@ -2299,7 +2056,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="12">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>75</v>
       </c>
@@ -2318,117 +2075,120 @@
     <cfRule type="duplicateValues" dxfId="0" priority="1"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
+  <dimension ref="A1:G8"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
-        <v>101</v>
+        <v>79</v>
       </c>
       <c r="B1" t="s">
         <v>47</v>
       </c>
       <c r="C1" t="s">
-        <v>109</v>
+        <v>83</v>
       </c>
       <c r="D1" t="s">
-        <v>142</v>
+        <v>103</v>
       </c>
       <c r="E1" t="s">
-        <v>119</v>
+        <v>89</v>
       </c>
       <c r="F1" t="s">
-        <v>124</v>
+        <v>94</v>
       </c>
       <c r="G1" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>102</v>
+        <v>80</v>
       </c>
       <c r="B2" t="s">
         <v>48</v>
       </c>
       <c r="C2" t="s">
-        <v>110</v>
+        <v>84</v>
       </c>
       <c r="D2" t="s">
-        <v>144</v>
+        <v>105</v>
       </c>
       <c r="E2" t="s">
-        <v>120</v>
+        <v>90</v>
       </c>
       <c r="F2" t="s">
-        <v>125</v>
+        <v>95</v>
       </c>
       <c r="G2" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="3">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>103</v>
+        <v>168</v>
       </c>
       <c r="B3" t="s">
-        <v>106</v>
+        <v>82</v>
       </c>
       <c r="C3" t="s">
-        <v>111</v>
+        <v>85</v>
       </c>
       <c r="D3" t="s">
-        <v>143</v>
+        <v>104</v>
       </c>
       <c r="E3" t="s">
-        <v>121</v>
+        <v>91</v>
       </c>
       <c r="F3" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="4">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>104</v>
+        <v>169</v>
       </c>
       <c r="E4" t="s">
-        <v>122</v>
+        <v>92</v>
       </c>
       <c r="F4" t="s">
-        <v>127</v>
-      </c>
-    </row>
-    <row r="5">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>81</v>
+      </c>
       <c r="E5" t="s">
-        <v>123</v>
+        <v>93</v>
       </c>
       <c r="F5" t="s">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="6">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
       <c r="F6" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="7">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
       <c r="F7" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="8">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
       <c r="F8" t="s">
-        <v>131</v>
+        <v>101</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
QC viability guard, header path fix, metadata update, remove CLAUDE.md from repo
- Pipeline: skip QC gracefully when samples too small (<2000 any QC, <5000 PeacoQC)
- Pipeline: render callout warning in report when QC is skipped
- Pipeline: remove time_channel_parameter from PeacoQC call
- marmot.R: point QMD at installed header path instead of copying into results folder
- Metadata xlsx updated (removed condaDir/parcScriptDir)
- Tests: 3 new QC skip tests, PeacoQC tests bumped to 5000 events
- CLAUDE.md removed from tracking, added to .gitignore

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/inst/pipeline/MARMOT_Metadata.xlsx
+++ b/inst/pipeline/MARMOT_Metadata.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10222"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10302"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/peterleary/Desktop/marmot/inst/pipeline/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A68404DC-9563-5B43-9B38-B62407FA469A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{181D54C2-38F3-C040-BE62-AA74A1B4FD71}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="6560" yWindow="4620" windowWidth="34560" windowHeight="20440" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="6560" yWindow="4620" windowWidth="34560" windowHeight="20440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Pipeline Settings" sheetId="3" r:id="rId1"/>
@@ -586,7 +586,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="9">
+  <fills count="10">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -635,8 +635,14 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC1FC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="12">
+  <borders count="11">
     <border>
       <left/>
       <right/>
@@ -753,15 +759,6 @@
       <bottom style="thin">
         <color indexed="64"/>
       </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
       <diagonal/>
     </border>
     <border>
@@ -841,18 +838,18 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="9" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="9" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -880,6 +877,12 @@
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <colors>
+    <mruColors>
+      <color rgb="FFFFC1FC"/>
+      <color rgb="FFFF8DF3"/>
+    </mruColors>
+  </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -1307,122 +1310,122 @@
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A11" s="14" t="s">
-        <v>142</v>
-      </c>
-      <c r="B11" s="15"/>
-      <c r="C11" s="16" t="s">
-        <v>143</v>
+      <c r="A11" s="29" t="s">
+        <v>166</v>
+      </c>
+      <c r="B11" s="29" t="s">
+        <v>140</v>
+      </c>
+      <c r="C11" s="30" t="s">
+        <v>167</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A12" s="14" t="s">
-        <v>144</v>
-      </c>
-      <c r="B12" s="15" t="s">
-        <v>140</v>
-      </c>
+        <v>142</v>
+      </c>
+      <c r="B12" s="15"/>
       <c r="C12" s="16" t="s">
-        <v>87</v>
+        <v>143</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A13" s="14" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="B13" s="15" t="s">
         <v>140</v>
       </c>
       <c r="C13" s="16" t="s">
-        <v>146</v>
+        <v>87</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A14" s="14" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="B14" s="15" t="s">
-        <v>148</v>
+        <v>140</v>
       </c>
       <c r="C14" s="16" t="s">
-        <v>149</v>
+        <v>146</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A15" s="14" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
       <c r="B15" s="15" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="C15" s="16" t="s">
-        <v>88</v>
+        <v>149</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A16" s="14" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="B16" s="15" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="C16" s="16" t="s">
-        <v>154</v>
+        <v>88</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A17" s="14" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="B17" s="15" t="s">
-        <v>156</v>
+        <v>153</v>
       </c>
       <c r="C17" s="16" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A18" s="14" t="s">
+        <v>155</v>
+      </c>
+      <c r="B18" s="15" t="s">
+        <v>156</v>
+      </c>
+      <c r="C18" s="16" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A19" s="14" t="s">
         <v>158</v>
       </c>
-      <c r="B18" s="15" t="s">
+      <c r="B19" s="15" t="s">
         <v>159</v>
       </c>
-      <c r="C18" s="16" t="s">
+      <c r="C19" s="16" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A19" s="17" t="s">
+    <row r="20" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A20" s="17" t="s">
         <v>160</v>
       </c>
-      <c r="B19" s="18" t="s">
+      <c r="B20" s="18" t="s">
         <v>161</v>
       </c>
-      <c r="C19" s="19" t="s">
+      <c r="C20" s="19" t="s">
         <v>162</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A20" s="20" t="s">
+    <row r="21" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A21" s="20" t="s">
         <v>163</v>
       </c>
-      <c r="B20" s="21" t="s">
+      <c r="B21" s="21" t="s">
         <v>164</v>
       </c>
-      <c r="C20" s="22" t="s">
+      <c r="C21" s="22" t="s">
         <v>165</v>
-      </c>
-    </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A21" s="25" t="s">
-        <v>166</v>
-      </c>
-      <c r="B21" s="25" t="s">
-        <v>140</v>
-      </c>
-      <c r="C21" s="26" t="s">
-        <v>167</v>
       </c>
     </row>
   </sheetData>
@@ -1452,19 +1455,19 @@
           <x14:formula1>
             <xm:f>Options!$G$1:$G$2</xm:f>
           </x14:formula1>
-          <xm:sqref>B10</xm:sqref>
+          <xm:sqref>B10:B11</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{EF0F4D8A-D969-2040-A7B2-4D843CC1D241}">
           <x14:formula1>
             <xm:f>Options!$E$1:$E$5</xm:f>
           </x14:formula1>
-          <xm:sqref>B17</xm:sqref>
+          <xm:sqref>B18</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{D6D0959A-58E3-6B40-9F0A-C50FD537F1F2}">
           <x14:formula1>
             <xm:f>Options!$F$1:$F$8</xm:f>
           </x14:formula1>
-          <xm:sqref>B18</xm:sqref>
+          <xm:sqref>B19</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{C81D77FB-D1A4-0B4C-B41A-E5791F351257}">
           <x14:formula1>
@@ -1476,19 +1479,19 @@
           <x14:formula1>
             <xm:f>Options!G1:G2</xm:f>
           </x14:formula1>
-          <xm:sqref>B12</xm:sqref>
+          <xm:sqref>B13</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{5D9B856C-01B5-4640-9249-FF510B93E1FC}">
           <x14:formula1>
             <xm:f>Options!G1:G2</xm:f>
           </x14:formula1>
-          <xm:sqref>B13</xm:sqref>
+          <xm:sqref>B14</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{93DD8684-4441-9741-BAB6-CBE45BFB25B6}">
           <x14:formula1>
             <xm:f>Options!G1:G2</xm:f>
           </x14:formula1>
-          <xm:sqref>B14</xm:sqref>
+          <xm:sqref>B15</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{ED65EFD9-012C-8E42-BE3B-3B16546394D0}">
           <x14:formula1>
@@ -1522,28 +1525,28 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="91" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="28" t="s">
+      <c r="A1" s="26" t="s">
         <v>16</v>
       </c>
-      <c r="B1" s="28" t="s">
+      <c r="B1" s="26" t="s">
         <v>53</v>
       </c>
-      <c r="C1" s="28" t="s">
+      <c r="C1" s="26" t="s">
         <v>0</v>
       </c>
-      <c r="D1" s="28" t="s">
+      <c r="D1" s="26" t="s">
         <v>21</v>
       </c>
-      <c r="E1" s="28" t="s">
+      <c r="E1" s="26" t="s">
         <v>20</v>
       </c>
-      <c r="F1" s="28" t="s">
+      <c r="F1" s="26" t="s">
         <v>1</v>
       </c>
-      <c r="G1" s="28" t="s">
+      <c r="G1" s="26" t="s">
         <v>2</v>
       </c>
-      <c r="H1" s="28" t="s">
+      <c r="H1" s="26" t="s">
         <v>23</v>
       </c>
     </row>
@@ -1563,7 +1566,7 @@
       <c r="E2" t="s">
         <v>47</v>
       </c>
-      <c r="F2" s="27">
+      <c r="F2" s="25">
         <v>2500</v>
       </c>
       <c r="G2" t="s">
@@ -1586,7 +1589,7 @@
       <c r="E3" t="s">
         <v>47</v>
       </c>
-      <c r="F3" s="27">
+      <c r="F3" s="25">
         <v>2500</v>
       </c>
       <c r="G3" t="s">
@@ -1603,7 +1606,7 @@
       <c r="E4" t="s">
         <v>47</v>
       </c>
-      <c r="F4" s="27">
+      <c r="F4" s="25">
         <v>2500</v>
       </c>
       <c r="G4" t="s">
@@ -1620,7 +1623,7 @@
       <c r="E5" t="s">
         <v>47</v>
       </c>
-      <c r="F5" s="27">
+      <c r="F5" s="25">
         <v>2500</v>
       </c>
       <c r="G5" t="s">
@@ -1637,7 +1640,7 @@
       <c r="E6" t="s">
         <v>47</v>
       </c>
-      <c r="F6" s="27">
+      <c r="F6" s="25">
         <v>2500</v>
       </c>
       <c r="G6" t="s">
@@ -1654,7 +1657,7 @@
       <c r="E7" t="s">
         <v>47</v>
       </c>
-      <c r="F7" s="27">
+      <c r="F7" s="25">
         <v>2500</v>
       </c>
       <c r="G7" t="s">
@@ -1671,7 +1674,7 @@
       <c r="E8" t="s">
         <v>47</v>
       </c>
-      <c r="F8" s="27">
+      <c r="F8" s="25">
         <v>2500</v>
       </c>
       <c r="G8" t="s">
@@ -1688,7 +1691,7 @@
       <c r="E9" t="s">
         <v>47</v>
       </c>
-      <c r="F9" s="27">
+      <c r="F9" s="25">
         <v>2500</v>
       </c>
       <c r="G9" t="s">
@@ -1705,7 +1708,7 @@
       <c r="E10" t="s">
         <v>48</v>
       </c>
-      <c r="F10" s="27">
+      <c r="F10" s="25">
         <v>2500</v>
       </c>
       <c r="G10" t="s">
@@ -1722,7 +1725,7 @@
       <c r="E11" t="s">
         <v>48</v>
       </c>
-      <c r="F11" s="27">
+      <c r="F11" s="25">
         <v>2500</v>
       </c>
       <c r="G11" t="s">
@@ -1736,7 +1739,7 @@
       <c r="E12" t="s">
         <v>47</v>
       </c>
-      <c r="F12" s="27">
+      <c r="F12" s="25">
         <v>2500</v>
       </c>
       <c r="G12" t="s">
@@ -1750,7 +1753,7 @@
       <c r="E13" t="s">
         <v>47</v>
       </c>
-      <c r="F13" s="27">
+      <c r="F13" s="25">
         <v>2500</v>
       </c>
     </row>
@@ -1761,7 +1764,7 @@
       <c r="E14" t="s">
         <v>47</v>
       </c>
-      <c r="F14" s="27">
+      <c r="F14" s="25">
         <v>2500</v>
       </c>
     </row>
@@ -1772,7 +1775,7 @@
       <c r="E15" t="s">
         <v>47</v>
       </c>
-      <c r="F15" s="27">
+      <c r="F15" s="25">
         <v>2500</v>
       </c>
     </row>
@@ -1783,7 +1786,7 @@
       <c r="E16" t="s">
         <v>47</v>
       </c>
-      <c r="F16" s="27">
+      <c r="F16" s="25">
         <v>2500</v>
       </c>
     </row>
@@ -1794,7 +1797,7 @@
       <c r="E17" t="s">
         <v>48</v>
       </c>
-      <c r="F17" s="27">
+      <c r="F17" s="25">
         <v>2500</v>
       </c>
     </row>
@@ -1805,7 +1808,7 @@
       <c r="E18" t="s">
         <v>48</v>
       </c>
-      <c r="F18" s="27">
+      <c r="F18" s="25">
         <v>2500</v>
       </c>
     </row>
@@ -1816,7 +1819,7 @@
       <c r="E19" t="s">
         <v>48</v>
       </c>
-      <c r="F19" s="27">
+      <c r="F19" s="25">
         <v>2500</v>
       </c>
     </row>
@@ -1827,7 +1830,7 @@
       <c r="E20" t="s">
         <v>48</v>
       </c>
-      <c r="F20" s="27">
+      <c r="F20" s="25">
         <v>2500</v>
       </c>
     </row>
@@ -1838,7 +1841,7 @@
       <c r="E21" t="s">
         <v>48</v>
       </c>
-      <c r="F21" s="27">
+      <c r="F21" s="25">
         <v>2500</v>
       </c>
     </row>
@@ -1849,7 +1852,7 @@
       <c r="E22" t="s">
         <v>48</v>
       </c>
-      <c r="F22" s="27">
+      <c r="F22" s="25">
         <v>2500</v>
       </c>
     </row>
@@ -1860,7 +1863,7 @@
       <c r="E23" t="s">
         <v>47</v>
       </c>
-      <c r="F23" s="27">
+      <c r="F23" s="25">
         <v>2500</v>
       </c>
     </row>
@@ -1871,7 +1874,7 @@
       <c r="E24" t="s">
         <v>48</v>
       </c>
-      <c r="F24" s="27">
+      <c r="F24" s="25">
         <v>2500</v>
       </c>
     </row>
@@ -1882,7 +1885,7 @@
       <c r="E25" t="s">
         <v>48</v>
       </c>
-      <c r="F25" s="27">
+      <c r="F25" s="25">
         <v>2500</v>
       </c>
     </row>
@@ -1903,16 +1906,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A1" s="29" t="s">
+      <c r="A1" s="27" t="s">
         <v>11</v>
       </c>
-      <c r="B1" s="29" t="s">
+      <c r="B1" s="27" t="s">
         <v>12</v>
       </c>
-      <c r="C1" s="29" t="s">
+      <c r="C1" s="27" t="s">
         <v>3</v>
       </c>
-      <c r="D1" s="30" t="s">
+      <c r="D1" s="28" t="s">
         <v>50</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Pipeline QC/DPI/DS fixes, Tauri marker pairs UI, Python DR runner
</commit_message>
<xml_diff>
--- a/inst/pipeline/MARMOT_Metadata.xlsx
+++ b/inst/pipeline/MARMOT_Metadata.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10302"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10404"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/peterleary/Desktop/marmot/inst/pipeline/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{181D54C2-38F3-C040-BE62-AA74A1B4FD71}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D2D89F80-4190-F74D-9BA0-278C2CB7F484}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="6560" yWindow="4620" windowWidth="34560" windowHeight="20440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="780" windowWidth="41120" windowHeight="24720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Pipeline Settings" sheetId="3" r:id="rId1"/>
@@ -27,12 +27,25 @@
     <definedName name="themeToUse">Options!$E$1:$E$5</definedName>
     <definedName name="viridisColour">Options!$F$1:$F$8</definedName>
   </definedNames>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="218" uniqueCount="170">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="220" uniqueCount="172">
   <si>
     <t>Conditions To Test</t>
   </si>
@@ -418,9 +431,6 @@
     <t>20 40 60</t>
   </si>
   <si>
-    <t>Number of knn/metacluster values to include in some of the visualisation, to see how over-/under-clustered you are. Space separated numbers, please.</t>
-  </si>
-  <si>
     <t>knn</t>
   </si>
   <si>
@@ -542,22 +552,23 @@
   </si>
   <si>
     <t>MfastPG</t>
+  </si>
+  <si>
+    <t>Mparc</t>
+  </si>
+  <si>
+    <t>Mpacmap</t>
+  </si>
+  <si>
+    <t>Number of knn/metacluster values to include in some of the visualisation, to see how over-/under-clustered you are. Space separated numbers, please. Please use odd numbers of Phenograph/PARC and even numbers for FlowSOM.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
-      <sz val="12"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="12"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -579,14 +590,34 @@
     </font>
     <font>
       <b/>
-      <sz val="22"/>
-      <color theme="1"/>
+      <sz val="16"/>
+      <color theme="0"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="16"/>
+      <color theme="0"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="16"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="14"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="10">
+  <fills count="12">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -631,18 +662,30 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.59999389629810485"/>
+        <fgColor rgb="FFFFC1FC"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFC1FC"/>
+        <fgColor theme="3"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="3" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0" tint="-4.9989318521683403E-2"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="11">
+  <borders count="21">
     <border>
       <left/>
       <right/>
@@ -680,21 +723,6 @@
       <left style="thin">
         <color indexed="64"/>
       </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
       <right/>
       <top style="thin">
         <color indexed="64"/>
@@ -772,6 +800,115 @@
         <color indexed="64"/>
       </top>
       <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
         <color indexed="64"/>
       </bottom>
       <diagonal/>
@@ -780,81 +917,82 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="34">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="11" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="11" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="10" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="11" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="10" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="11" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="11" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="7" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="10" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="7" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="11" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="10" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="2" fillId="9" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="9" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="2">
+  <dxfs count="3">
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -862,6 +1000,16 @@
       <fill>
         <patternFill>
           <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1194,243 +1342,243 @@
   <dimension ref="A1:C21"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="20.83203125" customWidth="1"/>
-    <col min="2" max="2" width="22.83203125" customWidth="1"/>
-    <col min="3" max="3" width="128.6640625" customWidth="1"/>
+    <col min="1" max="1" width="26.83203125" customWidth="1"/>
+    <col min="2" max="2" width="21.1640625" customWidth="1"/>
+    <col min="3" max="3" width="196" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A1" s="24" t="s">
+    <row r="1" spans="1:3" ht="21" x14ac:dyDescent="0.25">
+      <c r="A1" s="8" t="s">
         <v>114</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="8" t="s">
         <v>115</v>
       </c>
-      <c r="C1" s="23" t="s">
+      <c r="C1" s="9" t="s">
         <v>116</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A2" s="2" t="s">
+    <row r="2" spans="1:3" ht="19" x14ac:dyDescent="0.25">
+      <c r="A2" s="26" t="s">
         <v>117</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="B2" s="27" t="s">
         <v>118</v>
       </c>
-      <c r="C2" s="4" t="s">
+      <c r="C2" s="28" t="s">
         <v>119</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A3" s="5" t="s">
+    <row r="3" spans="1:3" ht="19" x14ac:dyDescent="0.25">
+      <c r="A3" s="21" t="s">
         <v>120</v>
       </c>
-      <c r="B3" s="6" t="s">
+      <c r="B3" s="16" t="s">
         <v>121</v>
       </c>
-      <c r="C3" s="7" t="s">
+      <c r="C3" s="22" t="s">
         <v>122</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A4" s="5" t="s">
+    <row r="4" spans="1:3" ht="19" x14ac:dyDescent="0.25">
+      <c r="A4" s="21" t="s">
         <v>123</v>
       </c>
-      <c r="B4" s="6" t="s">
+      <c r="B4" s="16" t="s">
         <v>124</v>
       </c>
-      <c r="C4" s="7" t="s">
+      <c r="C4" s="22" t="s">
         <v>125</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A5" s="5" t="s">
+    <row r="5" spans="1:3" ht="19" x14ac:dyDescent="0.25">
+      <c r="A5" s="21" t="s">
         <v>126</v>
       </c>
-      <c r="B5" s="6" t="s">
+      <c r="B5" s="16" t="s">
         <v>127</v>
       </c>
-      <c r="C5" s="7" t="s">
+      <c r="C5" s="22" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" ht="19" x14ac:dyDescent="0.25">
+      <c r="A6" s="23" t="s">
         <v>128</v>
       </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A6" s="5" t="s">
+      <c r="B6" s="24" t="s">
         <v>129</v>
       </c>
-      <c r="B6" s="6" t="s">
+      <c r="C6" s="25" t="s">
         <v>130</v>
       </c>
-      <c r="C6" s="7" t="s">
+    </row>
+    <row r="7" spans="1:3" ht="19" x14ac:dyDescent="0.25">
+      <c r="A7" s="19" t="s">
         <v>131</v>
       </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A7" s="8" t="s">
+      <c r="B7" s="20" t="s">
         <v>132</v>
       </c>
-      <c r="B7" s="9" t="s">
+      <c r="C7" s="29" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" ht="19" x14ac:dyDescent="0.25">
+      <c r="A8" s="23" t="s">
         <v>133</v>
       </c>
-      <c r="C7" s="10" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A8" s="8" t="s">
+      <c r="B8" s="24" t="s">
         <v>134</v>
       </c>
-      <c r="B8" s="9" t="s">
+      <c r="C8" s="30" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" ht="19" x14ac:dyDescent="0.25">
+      <c r="A9" s="19" t="s">
         <v>135</v>
       </c>
-      <c r="C8" s="10" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A9" s="11" t="s">
+      <c r="B9" s="20" t="s">
         <v>136</v>
       </c>
-      <c r="B9" s="12" t="s">
+      <c r="C9" s="31" t="s">
         <v>137</v>
       </c>
-      <c r="C9" s="13" t="s">
+    </row>
+    <row r="10" spans="1:3" ht="19" x14ac:dyDescent="0.25">
+      <c r="A10" s="23" t="s">
         <v>138</v>
       </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A10" s="11" t="s">
+      <c r="B10" s="24" t="s">
         <v>139</v>
       </c>
-      <c r="B10" s="12" t="s">
+      <c r="C10" s="32" t="s">
         <v>140</v>
       </c>
-      <c r="C10" s="13" t="s">
+    </row>
+    <row r="11" spans="1:3" ht="19" x14ac:dyDescent="0.25">
+      <c r="A11" s="26" t="s">
+        <v>165</v>
+      </c>
+      <c r="B11" s="27" t="s">
+        <v>139</v>
+      </c>
+      <c r="C11" s="33" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" ht="19" x14ac:dyDescent="0.25">
+      <c r="A12" s="15" t="s">
+        <v>143</v>
+      </c>
+      <c r="B12" s="16" t="s">
+        <v>139</v>
+      </c>
+      <c r="C12" s="13" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" ht="19" x14ac:dyDescent="0.25">
+      <c r="A13" s="15" t="s">
+        <v>144</v>
+      </c>
+      <c r="B13" s="16" t="s">
+        <v>139</v>
+      </c>
+      <c r="C13" s="13" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" ht="19" x14ac:dyDescent="0.25">
+      <c r="A14" s="15" t="s">
+        <v>146</v>
+      </c>
+      <c r="B14" s="16" t="s">
+        <v>147</v>
+      </c>
+      <c r="C14" s="13" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" ht="19" x14ac:dyDescent="0.25">
+      <c r="A15" s="15" t="s">
+        <v>149</v>
+      </c>
+      <c r="B15" s="16" t="s">
+        <v>150</v>
+      </c>
+      <c r="C15" s="13" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" ht="19" x14ac:dyDescent="0.25">
+      <c r="A16" s="15" t="s">
+        <v>151</v>
+      </c>
+      <c r="B16" s="16" t="s">
+        <v>152</v>
+      </c>
+      <c r="C16" s="13" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" ht="19" x14ac:dyDescent="0.25">
+      <c r="A17" s="15" t="s">
         <v>141</v>
       </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A11" s="29" t="s">
-        <v>166</v>
-      </c>
-      <c r="B11" s="29" t="s">
-        <v>140</v>
-      </c>
-      <c r="C11" s="30" t="s">
-        <v>167</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A12" s="14" t="s">
+      <c r="B17" s="16"/>
+      <c r="C17" s="13" t="s">
         <v>142</v>
       </c>
-      <c r="B12" s="15"/>
-      <c r="C12" s="16" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A13" s="14" t="s">
-        <v>144</v>
-      </c>
-      <c r="B13" s="15" t="s">
-        <v>140</v>
-      </c>
-      <c r="C13" s="16" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A14" s="14" t="s">
-        <v>145</v>
-      </c>
-      <c r="B14" s="15" t="s">
-        <v>140</v>
-      </c>
-      <c r="C14" s="16" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A15" s="14" t="s">
-        <v>147</v>
-      </c>
-      <c r="B15" s="15" t="s">
-        <v>148</v>
-      </c>
-      <c r="C15" s="16" t="s">
-        <v>149</v>
-      </c>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A16" s="14" t="s">
-        <v>150</v>
-      </c>
-      <c r="B16" s="15" t="s">
-        <v>151</v>
-      </c>
-      <c r="C16" s="16" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A17" s="14" t="s">
-        <v>152</v>
-      </c>
-      <c r="B17" s="15" t="s">
-        <v>153</v>
-      </c>
-      <c r="C17" s="16" t="s">
+    </row>
+    <row r="18" spans="1:3" ht="19" x14ac:dyDescent="0.25">
+      <c r="A18" s="15" t="s">
         <v>154</v>
       </c>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A18" s="14" t="s">
+      <c r="B18" s="16" t="s">
         <v>155</v>
       </c>
-      <c r="B18" s="15" t="s">
+      <c r="C18" s="13" t="s">
         <v>156</v>
       </c>
-      <c r="C18" s="16" t="s">
+    </row>
+    <row r="19" spans="1:3" ht="20" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A19" s="17" t="s">
         <v>157</v>
       </c>
-    </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A19" s="14" t="s">
+      <c r="B19" s="18" t="s">
         <v>158</v>
       </c>
-      <c r="B19" s="15" t="s">
+      <c r="C19" s="14" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A20" s="10" t="s">
         <v>159</v>
       </c>
-      <c r="C19" s="16" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="20" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
-      <c r="A20" s="17" t="s">
+      <c r="B20" s="11" t="s">
         <v>160</v>
       </c>
-      <c r="B20" s="18" t="s">
+      <c r="C20" s="12" t="s">
         <v>161</v>
       </c>
-      <c r="C20" s="19" t="s">
+    </row>
+    <row r="21" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A21" s="1" t="s">
         <v>162</v>
       </c>
-    </row>
-    <row r="21" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
-      <c r="A21" s="20" t="s">
+      <c r="B21" s="2" t="s">
         <v>163</v>
       </c>
-      <c r="B21" s="21" t="s">
+      <c r="C21" s="3" t="s">
         <v>164</v>
-      </c>
-      <c r="C21" s="22" t="s">
-        <v>165</v>
       </c>
     </row>
   </sheetData>
   <conditionalFormatting sqref="B3">
-    <cfRule type="expression" dxfId="1" priority="1">
+    <cfRule type="expression" dxfId="2" priority="1">
       <formula>ISBLANK(A3)</formula>
     </cfRule>
   </conditionalFormatting>
@@ -1479,19 +1627,19 @@
           <x14:formula1>
             <xm:f>Options!G1:G2</xm:f>
           </x14:formula1>
-          <xm:sqref>B13</xm:sqref>
+          <xm:sqref>B12</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{5D9B856C-01B5-4640-9249-FF510B93E1FC}">
           <x14:formula1>
             <xm:f>Options!G1:G2</xm:f>
           </x14:formula1>
-          <xm:sqref>B14</xm:sqref>
+          <xm:sqref>B13</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{93DD8684-4441-9741-BAB6-CBE45BFB25B6}">
           <x14:formula1>
             <xm:f>Options!G1:G2</xm:f>
           </x14:formula1>
-          <xm:sqref>B15</xm:sqref>
+          <xm:sqref>B14</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{ED65EFD9-012C-8E42-BE3B-3B16546394D0}">
           <x14:formula1>
@@ -1524,29 +1672,29 @@
     <col min="8" max="8" width="26" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="91" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="26" t="s">
+    <row r="1" spans="1:8" ht="54" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A1" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="B1" s="26" t="s">
+      <c r="B1" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="C1" s="26" t="s">
+      <c r="C1" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="D1" s="26" t="s">
+      <c r="D1" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="E1" s="26" t="s">
+      <c r="E1" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="F1" s="26" t="s">
+      <c r="F1" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="G1" s="26" t="s">
+      <c r="G1" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="H1" s="26" t="s">
+      <c r="H1" s="5" t="s">
         <v>23</v>
       </c>
     </row>
@@ -1566,7 +1714,7 @@
       <c r="E2" t="s">
         <v>47</v>
       </c>
-      <c r="F2" s="25">
+      <c r="F2" s="4">
         <v>2500</v>
       </c>
       <c r="G2" t="s">
@@ -1589,7 +1737,7 @@
       <c r="E3" t="s">
         <v>47</v>
       </c>
-      <c r="F3" s="25">
+      <c r="F3" s="4">
         <v>2500</v>
       </c>
       <c r="G3" t="s">
@@ -1606,7 +1754,7 @@
       <c r="E4" t="s">
         <v>47</v>
       </c>
-      <c r="F4" s="25">
+      <c r="F4" s="4">
         <v>2500</v>
       </c>
       <c r="G4" t="s">
@@ -1623,7 +1771,7 @@
       <c r="E5" t="s">
         <v>47</v>
       </c>
-      <c r="F5" s="25">
+      <c r="F5" s="4">
         <v>2500</v>
       </c>
       <c r="G5" t="s">
@@ -1640,7 +1788,7 @@
       <c r="E6" t="s">
         <v>47</v>
       </c>
-      <c r="F6" s="25">
+      <c r="F6" s="4">
         <v>2500</v>
       </c>
       <c r="G6" t="s">
@@ -1657,7 +1805,7 @@
       <c r="E7" t="s">
         <v>47</v>
       </c>
-      <c r="F7" s="25">
+      <c r="F7" s="4">
         <v>2500</v>
       </c>
       <c r="G7" t="s">
@@ -1674,7 +1822,7 @@
       <c r="E8" t="s">
         <v>47</v>
       </c>
-      <c r="F8" s="25">
+      <c r="F8" s="4">
         <v>2500</v>
       </c>
       <c r="G8" t="s">
@@ -1691,7 +1839,7 @@
       <c r="E9" t="s">
         <v>47</v>
       </c>
-      <c r="F9" s="25">
+      <c r="F9" s="4">
         <v>2500</v>
       </c>
       <c r="G9" t="s">
@@ -1708,7 +1856,7 @@
       <c r="E10" t="s">
         <v>48</v>
       </c>
-      <c r="F10" s="25">
+      <c r="F10" s="4">
         <v>2500</v>
       </c>
       <c r="G10" t="s">
@@ -1725,7 +1873,7 @@
       <c r="E11" t="s">
         <v>48</v>
       </c>
-      <c r="F11" s="25">
+      <c r="F11" s="4">
         <v>2500</v>
       </c>
       <c r="G11" t="s">
@@ -1739,7 +1887,7 @@
       <c r="E12" t="s">
         <v>47</v>
       </c>
-      <c r="F12" s="25">
+      <c r="F12" s="4">
         <v>2500</v>
       </c>
       <c r="G12" t="s">
@@ -1753,7 +1901,7 @@
       <c r="E13" t="s">
         <v>47</v>
       </c>
-      <c r="F13" s="25">
+      <c r="F13" s="4">
         <v>2500</v>
       </c>
     </row>
@@ -1764,7 +1912,7 @@
       <c r="E14" t="s">
         <v>47</v>
       </c>
-      <c r="F14" s="25">
+      <c r="F14" s="4">
         <v>2500</v>
       </c>
     </row>
@@ -1775,7 +1923,7 @@
       <c r="E15" t="s">
         <v>47</v>
       </c>
-      <c r="F15" s="25">
+      <c r="F15" s="4">
         <v>2500</v>
       </c>
     </row>
@@ -1786,7 +1934,7 @@
       <c r="E16" t="s">
         <v>47</v>
       </c>
-      <c r="F16" s="25">
+      <c r="F16" s="4">
         <v>2500</v>
       </c>
     </row>
@@ -1797,7 +1945,7 @@
       <c r="E17" t="s">
         <v>48</v>
       </c>
-      <c r="F17" s="25">
+      <c r="F17" s="4">
         <v>2500</v>
       </c>
     </row>
@@ -1808,7 +1956,7 @@
       <c r="E18" t="s">
         <v>48</v>
       </c>
-      <c r="F18" s="25">
+      <c r="F18" s="4">
         <v>2500</v>
       </c>
     </row>
@@ -1819,7 +1967,7 @@
       <c r="E19" t="s">
         <v>48</v>
       </c>
-      <c r="F19" s="25">
+      <c r="F19" s="4">
         <v>2500</v>
       </c>
     </row>
@@ -1830,7 +1978,7 @@
       <c r="E20" t="s">
         <v>48</v>
       </c>
-      <c r="F20" s="25">
+      <c r="F20" s="4">
         <v>2500</v>
       </c>
     </row>
@@ -1841,7 +1989,7 @@
       <c r="E21" t="s">
         <v>48</v>
       </c>
-      <c r="F21" s="25">
+      <c r="F21" s="4">
         <v>2500</v>
       </c>
     </row>
@@ -1852,7 +2000,7 @@
       <c r="E22" t="s">
         <v>48</v>
       </c>
-      <c r="F22" s="25">
+      <c r="F22" s="4">
         <v>2500</v>
       </c>
     </row>
@@ -1863,7 +2011,7 @@
       <c r="E23" t="s">
         <v>47</v>
       </c>
-      <c r="F23" s="25">
+      <c r="F23" s="4">
         <v>2500</v>
       </c>
     </row>
@@ -1874,7 +2022,7 @@
       <c r="E24" t="s">
         <v>48</v>
       </c>
-      <c r="F24" s="25">
+      <c r="F24" s="4">
         <v>2500</v>
       </c>
     </row>
@@ -1885,7 +2033,7 @@
       <c r="E25" t="s">
         <v>48</v>
       </c>
-      <c r="F25" s="25">
+      <c r="F25" s="4">
         <v>2500</v>
       </c>
     </row>
@@ -1903,19 +2051,20 @@
     <col min="1" max="1" width="72.5" customWidth="1"/>
     <col min="2" max="2" width="18" customWidth="1"/>
     <col min="3" max="3" width="19.6640625" customWidth="1"/>
+    <col min="4" max="4" width="17.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A1" s="27" t="s">
+    <row r="1" spans="1:4" ht="21" x14ac:dyDescent="0.25">
+      <c r="A1" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="B1" s="27" t="s">
+      <c r="B1" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="C1" s="27" t="s">
+      <c r="C1" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="D1" s="28" t="s">
+      <c r="D1" s="7" t="s">
         <v>50</v>
       </c>
     </row>
@@ -2074,8 +2223,8 @@
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="B2:B12">
-    <cfRule type="duplicateValues" dxfId="0" priority="1"/>
+  <conditionalFormatting sqref="C2:C59">
+    <cfRule type="uniqueValues" dxfId="1" priority="1"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
@@ -2135,7 +2284,7 @@
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="B3" t="s">
         <v>82</v>
@@ -2155,7 +2304,10 @@
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>169</v>
+        <v>168</v>
+      </c>
+      <c r="C4" t="s">
+        <v>170</v>
       </c>
       <c r="E4" t="s">
         <v>92</v>
@@ -2176,6 +2328,9 @@
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
+        <v>169</v>
+      </c>
       <c r="F6" t="s">
         <v>99</v>
       </c>

</xml_diff>

<commit_message>
Pipeline: strict FCS matching, Windows RAM fallback, diagnostic log
- Strict basename equality between md$file_name and files in fcsDir.
  Missing file is fatal with a clear message; extras on disk are ignored.
  Kills the `.fcs.fcs` substring-match class of silent sample drops.
- Windows RAM probe drops `wmic` (deprecated on 11+). Emits a loud
  warning and falls back to user-declared ramPerCore x nCores.
- New ambient R_files/marmot_run_log.json: shape-only diagnostic log
  written progressively through rendering. Captures system, package
  versions, settings, data/clustering/DA/DS shape summaries, and
  render status. No cell values, no sample/condition labels —
  safe to attach to bug reports.
- Minor metadata.xlsx template tweak.
</commit_message>
<xml_diff>
--- a/inst/pipeline/MARMOT_Metadata.xlsx
+++ b/inst/pipeline/MARMOT_Metadata.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10404"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10412"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/peterleary/Desktop/marmot/inst/pipeline/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D2D89F80-4190-F74D-9BA0-278C2CB7F484}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{51A8F6DD-1742-1D4F-8BEC-9535FB5B8EBE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="780" windowWidth="41120" windowHeight="24720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -45,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="220" uniqueCount="172">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="219" uniqueCount="171">
   <si>
     <t>Conditions To Test</t>
   </si>
@@ -384,9 +384,6 @@
   </si>
   <si>
     <t>NK-Tcells: TCRb NK1.1</t>
-  </si>
-  <si>
-    <t>NK Cells: NK1.1+ CD3-</t>
   </si>
   <si>
     <t>Variable</t>
@@ -950,7 +947,7 @@
     <xf numFmtId="0" fontId="6" fillId="11" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="11" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -992,17 +989,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="3">
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="2">
     <dxf>
       <font>
         <color rgb="FF006100"/>
@@ -1349,76 +1336,76 @@
   <sheetData>
     <row r="1" spans="1:3" ht="21" x14ac:dyDescent="0.25">
       <c r="A1" s="8" t="s">
+        <v>113</v>
+      </c>
+      <c r="B1" s="8" t="s">
         <v>114</v>
       </c>
-      <c r="B1" s="8" t="s">
+      <c r="C1" s="9" t="s">
         <v>115</v>
-      </c>
-      <c r="C1" s="9" t="s">
-        <v>116</v>
       </c>
     </row>
     <row r="2" spans="1:3" ht="19" x14ac:dyDescent="0.25">
       <c r="A2" s="26" t="s">
+        <v>116</v>
+      </c>
+      <c r="B2" s="27" t="s">
         <v>117</v>
       </c>
-      <c r="B2" s="27" t="s">
+      <c r="C2" s="28" t="s">
         <v>118</v>
-      </c>
-      <c r="C2" s="28" t="s">
-        <v>119</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="19" x14ac:dyDescent="0.25">
       <c r="A3" s="21" t="s">
+        <v>119</v>
+      </c>
+      <c r="B3" s="16" t="s">
         <v>120</v>
       </c>
-      <c r="B3" s="16" t="s">
+      <c r="C3" s="22" t="s">
         <v>121</v>
-      </c>
-      <c r="C3" s="22" t="s">
-        <v>122</v>
       </c>
     </row>
     <row r="4" spans="1:3" ht="19" x14ac:dyDescent="0.25">
       <c r="A4" s="21" t="s">
+        <v>122</v>
+      </c>
+      <c r="B4" s="16" t="s">
         <v>123</v>
       </c>
-      <c r="B4" s="16" t="s">
+      <c r="C4" s="22" t="s">
         <v>124</v>
-      </c>
-      <c r="C4" s="22" t="s">
-        <v>125</v>
       </c>
     </row>
     <row r="5" spans="1:3" ht="19" x14ac:dyDescent="0.25">
       <c r="A5" s="21" t="s">
+        <v>125</v>
+      </c>
+      <c r="B5" s="16" t="s">
         <v>126</v>
       </c>
-      <c r="B5" s="16" t="s">
-        <v>127</v>
-      </c>
       <c r="C5" s="22" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
     </row>
     <row r="6" spans="1:3" ht="19" x14ac:dyDescent="0.25">
       <c r="A6" s="23" t="s">
+        <v>127</v>
+      </c>
+      <c r="B6" s="24" t="s">
         <v>128</v>
       </c>
-      <c r="B6" s="24" t="s">
+      <c r="C6" s="25" t="s">
         <v>129</v>
-      </c>
-      <c r="C6" s="25" t="s">
-        <v>130</v>
       </c>
     </row>
     <row r="7" spans="1:3" ht="19" x14ac:dyDescent="0.25">
       <c r="A7" s="19" t="s">
+        <v>130</v>
+      </c>
+      <c r="B7" s="20" t="s">
         <v>131</v>
-      </c>
-      <c r="B7" s="20" t="s">
-        <v>132</v>
       </c>
       <c r="C7" s="29" t="s">
         <v>86</v>
@@ -1426,54 +1413,54 @@
     </row>
     <row r="8" spans="1:3" ht="19" x14ac:dyDescent="0.25">
       <c r="A8" s="23" t="s">
+        <v>132</v>
+      </c>
+      <c r="B8" s="24" t="s">
         <v>133</v>
       </c>
-      <c r="B8" s="24" t="s">
-        <v>134</v>
-      </c>
       <c r="C8" s="30" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
     <row r="9" spans="1:3" ht="19" x14ac:dyDescent="0.25">
       <c r="A9" s="19" t="s">
+        <v>134</v>
+      </c>
+      <c r="B9" s="20" t="s">
         <v>135</v>
       </c>
-      <c r="B9" s="20" t="s">
+      <c r="C9" s="31" t="s">
         <v>136</v>
-      </c>
-      <c r="C9" s="31" t="s">
-        <v>137</v>
       </c>
     </row>
     <row r="10" spans="1:3" ht="19" x14ac:dyDescent="0.25">
       <c r="A10" s="23" t="s">
+        <v>137</v>
+      </c>
+      <c r="B10" s="24" t="s">
         <v>138</v>
       </c>
-      <c r="B10" s="24" t="s">
+      <c r="C10" s="32" t="s">
         <v>139</v>
-      </c>
-      <c r="C10" s="32" t="s">
-        <v>140</v>
       </c>
     </row>
     <row r="11" spans="1:3" ht="19" x14ac:dyDescent="0.25">
       <c r="A11" s="26" t="s">
+        <v>164</v>
+      </c>
+      <c r="B11" s="27" t="s">
+        <v>138</v>
+      </c>
+      <c r="C11" s="33" t="s">
         <v>165</v>
-      </c>
-      <c r="B11" s="27" t="s">
-        <v>139</v>
-      </c>
-      <c r="C11" s="33" t="s">
-        <v>166</v>
       </c>
     </row>
     <row r="12" spans="1:3" ht="19" x14ac:dyDescent="0.25">
       <c r="A12" s="15" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="B12" s="16" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="C12" s="13" t="s">
         <v>87</v>
@@ -1481,32 +1468,32 @@
     </row>
     <row r="13" spans="1:3" ht="19" x14ac:dyDescent="0.25">
       <c r="A13" s="15" t="s">
+        <v>143</v>
+      </c>
+      <c r="B13" s="16" t="s">
+        <v>138</v>
+      </c>
+      <c r="C13" s="13" t="s">
         <v>144</v>
-      </c>
-      <c r="B13" s="16" t="s">
-        <v>139</v>
-      </c>
-      <c r="C13" s="13" t="s">
-        <v>145</v>
       </c>
     </row>
     <row r="14" spans="1:3" ht="19" x14ac:dyDescent="0.25">
       <c r="A14" s="15" t="s">
+        <v>145</v>
+      </c>
+      <c r="B14" s="16" t="s">
         <v>146</v>
       </c>
-      <c r="B14" s="16" t="s">
+      <c r="C14" s="13" t="s">
         <v>147</v>
-      </c>
-      <c r="C14" s="13" t="s">
-        <v>148</v>
       </c>
     </row>
     <row r="15" spans="1:3" ht="19" x14ac:dyDescent="0.25">
       <c r="A15" s="15" t="s">
+        <v>148</v>
+      </c>
+      <c r="B15" s="16" t="s">
         <v>149</v>
-      </c>
-      <c r="B15" s="16" t="s">
-        <v>150</v>
       </c>
       <c r="C15" s="13" t="s">
         <v>88</v>
@@ -1514,41 +1501,41 @@
     </row>
     <row r="16" spans="1:3" ht="19" x14ac:dyDescent="0.25">
       <c r="A16" s="15" t="s">
+        <v>150</v>
+      </c>
+      <c r="B16" s="16" t="s">
         <v>151</v>
       </c>
-      <c r="B16" s="16" t="s">
+      <c r="C16" s="13" t="s">
         <v>152</v>
-      </c>
-      <c r="C16" s="13" t="s">
-        <v>153</v>
       </c>
     </row>
     <row r="17" spans="1:3" ht="19" x14ac:dyDescent="0.25">
       <c r="A17" s="15" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="B17" s="16"/>
       <c r="C17" s="13" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
     </row>
     <row r="18" spans="1:3" ht="19" x14ac:dyDescent="0.25">
       <c r="A18" s="15" t="s">
+        <v>153</v>
+      </c>
+      <c r="B18" s="16" t="s">
         <v>154</v>
       </c>
-      <c r="B18" s="16" t="s">
+      <c r="C18" s="13" t="s">
         <v>155</v>
-      </c>
-      <c r="C18" s="13" t="s">
-        <v>156</v>
       </c>
     </row>
     <row r="19" spans="1:3" ht="20" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A19" s="17" t="s">
+        <v>156</v>
+      </c>
+      <c r="B19" s="18" t="s">
         <v>157</v>
-      </c>
-      <c r="B19" s="18" t="s">
-        <v>158</v>
       </c>
       <c r="C19" s="14" t="s">
         <v>102</v>
@@ -1556,29 +1543,29 @@
     </row>
     <row r="20" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
       <c r="A20" s="10" t="s">
+        <v>158</v>
+      </c>
+      <c r="B20" s="11" t="s">
         <v>159</v>
       </c>
-      <c r="B20" s="11" t="s">
+      <c r="C20" s="12" t="s">
         <v>160</v>
-      </c>
-      <c r="C20" s="12" t="s">
-        <v>161</v>
       </c>
     </row>
     <row r="21" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
       <c r="A21" s="1" t="s">
+        <v>161</v>
+      </c>
+      <c r="B21" s="2" t="s">
         <v>162</v>
       </c>
-      <c r="B21" s="2" t="s">
+      <c r="C21" s="3" t="s">
         <v>163</v>
-      </c>
-      <c r="C21" s="3" t="s">
-        <v>164</v>
       </c>
     </row>
   </sheetData>
   <conditionalFormatting sqref="B3">
-    <cfRule type="expression" dxfId="2" priority="1">
+    <cfRule type="expression" dxfId="1" priority="1">
       <formula>ISBLANK(A3)</formula>
     </cfRule>
   </conditionalFormatting>
@@ -1862,9 +1849,6 @@
       <c r="G10" t="s">
         <v>10</v>
       </c>
-      <c r="H10" t="s">
-        <v>113</v>
-      </c>
     </row>
     <row r="11" spans="1:8" ht="19" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D11" t="s">
@@ -2224,7 +2208,7 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="C2:C59">
-    <cfRule type="uniqueValues" dxfId="1" priority="1"/>
+    <cfRule type="uniqueValues" dxfId="0" priority="1"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
@@ -2284,7 +2268,7 @@
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="B3" t="s">
         <v>82</v>
@@ -2304,10 +2288,10 @@
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="C4" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="E4" t="s">
         <v>92</v>
@@ -2329,7 +2313,7 @@
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="F6" t="s">
         <v>99</v>

</xml_diff>